<commit_message>
add pasture beef MMS
</commit_message>
<xml_diff>
--- a/Excel/4_1_ManureManagement_Feedlot_WIP_v04.xlsx
+++ b/Excel/4_1_ManureManagement_Feedlot_WIP_v04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6732AC43-75F1-44F1-80DC-705245AF9A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868BFF59-BF2F-4C1C-A1C3-6B773F8C5B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="630" yWindow="210" windowWidth="37755" windowHeight="20445" firstSheet="7" activeTab="9" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="630" yWindow="210" windowWidth="37755" windowHeight="20445" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -465,7 +465,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="345">
   <si>
     <t>Home</t>
   </si>
@@ -1658,18 +1658,12 @@
     <t>CO2-e unit</t>
   </si>
   <si>
-    <t>This feedlot</t>
-  </si>
-  <si>
     <t>Manure nitrogen sold</t>
   </si>
   <si>
     <t>Scope 3 (downstream)</t>
   </si>
   <si>
-    <t>Crops or pasture that use manure as fertiliser</t>
-  </si>
-  <si>
     <t>Amount of N in manure</t>
   </si>
   <si>
@@ -1685,9 +1679,6 @@
     <t>Manure nitrogen deposited on farm soils as fertiliser for other farm enterpsies (eg crops)</t>
   </si>
   <si>
-    <t>Manure nitrogen deposited on farm soils with no other purpose (aka waste)</t>
-  </si>
-  <si>
     <t>15.13.1.1 (1), 5.2.2.1 (1), 5.4.1.3 (1, 2), 5.5.1.1 (1, 3)</t>
   </si>
   <si>
@@ -1719,6 +1710,21 @@
   </si>
   <si>
     <t>EFPRP</t>
+  </si>
+  <si>
+    <t>Applied to farm soils as fertiliser for other enterprises (eg: crops)</t>
+  </si>
+  <si>
+    <t>apply queensland</t>
+  </si>
+  <si>
+    <t>use vic</t>
+  </si>
+  <si>
+    <t>Manure nitrogen deposited on farm soils (excluding farm fertiliser use)</t>
+  </si>
+  <si>
+    <t>Scope 1 - This feedlot</t>
   </si>
 </sst>
 </file>
@@ -2684,7 +2690,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="40" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -3068,6 +3074,9 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="8" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="65">
     <cellStyle name="Alert" xfId="62" xr:uid="{34EFE908-8095-4010-8F93-8CFE88055637}"/>
@@ -3137,6 +3146,246 @@
     <cellStyle name="Unit total" xfId="26" xr:uid="{65428923-3DAD-47B6-8DDF-0EBD05E7C55B}"/>
   </cellStyles>
   <dxfs count="59">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3618,246 +3867,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -10719,34 +10728,34 @@
     <tableColumn id="1" xr3:uid="{3885FE93-299E-44EB-B503-99C305BD6F41}" name="Treatment stage T">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D0E12F95-AC29-47D0-913A-0A0B02931616}" name="MMS m" dataDxfId="46" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{D0E12F95-AC29-47D0-913A-0A0B02931616}" name="MMS m" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E17BE7AB-8FAD-4B5C-9F86-E70E6A00B9B1}" name="NSW" dataDxfId="45" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{E17BE7AB-8FAD-4B5C-9F86-E70E6A00B9B1}" name="NSW" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D4C6F922-2719-4479-B7CC-26C5286F73ED}" name="ACT" dataDxfId="44" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{D4C6F922-2719-4479-B7CC-26C5286F73ED}" name="ACT" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5034DCA1-F046-43BC-A94F-832832E6D634}" name="QLD" dataDxfId="43" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5034DCA1-F046-43BC-A94F-832832E6D634}" name="QLD" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="4" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="40" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="3" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="39" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="2" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="38" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="1" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="37" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="0" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -10862,49 +10871,49 @@
     <tableColumn id="1" xr3:uid="{29672771-6091-4FA5-86EA-395E240FF5D2}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{7E0CB869-00AE-4755-8478-34C0A24DACCC}" name="MAT" totalsRowDxfId="18" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{7E0CB869-00AE-4755-8478-34C0A24DACCC}" name="MAT" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EEBB7F36-38AB-43CA-89EE-CBF9D2B12C70}" name="MAP" totalsRowDxfId="17" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{EEBB7F36-38AB-43CA-89EE-CBF9D2B12C70}" name="MAP" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{3010F3BA-675E-4D83-9AAD-FBE9EC6F9CF0}" name="Frost days per year" totalsRowDxfId="16" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{3010F3BA-675E-4D83-9AAD-FBE9EC6F9CF0}" name="Frost days per year" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{3F1B2FE9-64D5-41E9-9332-E943400478C4}" name="Elevation" totalsRowDxfId="15" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{3F1B2FE9-64D5-41E9-9332-E943400478C4}" name="Elevation" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{C4BB9839-93FF-42DA-A517-F34E10C70484}" name="MAP:PET" totalsRowDxfId="14" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{C4BB9839-93FF-42DA-A517-F34E10C70484}" name="MAP:PET" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{A01F6B36-D801-484C-A91E-3EFD0F4A77C0}" name="Min temp" totalsRowDxfId="13" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{A01F6B36-D801-484C-A91E-3EFD0F4A77C0}" name="Min temp" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{033C9484-1852-4D2B-88A9-02D24D40BB22}" name="Max temp" totalsRowDxfId="12" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{033C9484-1852-4D2B-88A9-02D24D40BB22}" name="Max temp" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{C54AFCDF-470B-41E8-8CB5-A1938A000F27}" name="Min rainfall" totalsRowDxfId="11" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{C54AFCDF-470B-41E8-8CB5-A1938A000F27}" name="Min rainfall" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{E235B24A-0205-4131-BBC7-FD5B69336BB5}" name="Max rainfall" totalsRowDxfId="10" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{E235B24A-0205-4131-BBC7-FD5B69336BB5}" name="Max rainfall" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{2236A619-E104-4738-8E09-41B8930DF78A}" name="Min frost days" totalsRowDxfId="9" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{2236A619-E104-4738-8E09-41B8930DF78A}" name="Min frost days" totalsRowDxfId="19" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{85D18FF3-E59D-404A-A2E0-032D9A5E0B84}" name="Max frost days" totalsRowDxfId="8" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{85D18FF3-E59D-404A-A2E0-032D9A5E0B84}" name="Max frost days" totalsRowDxfId="18" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{82A7ECE5-EF70-4355-AA39-B204B086F753}" name="Min elevation" totalsRowDxfId="7" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{82A7ECE5-EF70-4355-AA39-B204B086F753}" name="Min elevation" totalsRowDxfId="17" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{D75C68D2-6308-4B32-BFEC-DFF390DB8E53}" name="Max elevation" totalsRowDxfId="6" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{D75C68D2-6308-4B32-BFEC-DFF390DB8E53}" name="Max elevation" totalsRowDxfId="16" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{36486A17-D0A0-48BD-A954-F404E9596B7F}" name="Min MAP:PET" totalsRowDxfId="5" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{36486A17-D0A0-48BD-A954-F404E9596B7F}" name="Min MAP:PET" totalsRowDxfId="15" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{99A2031C-68A9-4CB7-9470-3CF073E8938E}" name="Max MAP:PET" totalsRowDxfId="4" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{99A2031C-68A9-4CB7-9470-3CF073E8938E}" name="Max MAP:PET" totalsRowDxfId="14" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -10922,7 +10931,7 @@
     <tableColumn id="1" xr3:uid="{2BBF6521-99F9-49EC-9C13-C6835493D245}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0DDE2867-2EF4-48CD-8D28-92B0EFFA35E5}" name="Wet or Dry Zone" totalsRowDxfId="3" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{0DDE2867-2EF4-48CD-8D28-92B0EFFA35E5}" name="Wet or Dry Zone" totalsRowDxfId="13" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11026,7 +11035,7 @@
   </autoFilter>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{F2B173A3-CADE-4DCA-988D-39EE2392D8DB}" name="MMS"/>
-    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="36" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="46" dataCellStyle="Content normal"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11042,7 +11051,7 @@
     <tableColumn id="1" xr3:uid="{7CC796C2-63D2-47F7-9053-D908618080F5}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DAA00D67-052D-437D-8304-FCF408B01074}" name="FracWET" dataDxfId="2">
+    <tableColumn id="2" xr3:uid="{DAA00D67-052D-437D-8304-FCF408B01074}" name="FracWET" dataDxfId="12">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11090,7 +11099,7 @@
     <tableColumn id="1" xr3:uid="{61DBB82B-3A6D-419F-8985-5F50A33AD54D}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{64F1A8DC-1528-499D-8C77-81E69EE8003E}" name="FracWET" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{64F1A8DC-1528-499D-8C77-81E69EE8003E}" name="FracWET" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11108,7 +11117,7 @@
     <tableColumn id="1" xr3:uid="{AE0190D4-8B38-4D11-A70F-AF75E033ACD3}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{32442D06-ACE7-48E5-A599-0F379CCEDA2A}" name="EFPRP" dataDxfId="0" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{32442D06-ACE7-48E5-A599-0F379CCEDA2A}" name="EFPRP" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11153,22 +11162,22 @@
     <tableColumn id="1" xr3:uid="{FDCB848C-205F-48EA-BACF-F54BCD324E05}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="45" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="44" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="33" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="43" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="32" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="42" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="41" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="40" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11191,22 +11200,22 @@
     <tableColumn id="1" xr3:uid="{96F6B4E3-E1EE-445F-9BCE-628B89FC3727}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="39" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="28" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="38" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="37" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="36" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="25" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="24" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11224,7 +11233,7 @@
     <tableColumn id="1" xr3:uid="{9D472457-4D8B-44ED-9567-B889D058C2F1}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="23" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11244,13 +11253,13 @@
     <tableColumn id="1" xr3:uid="{C80C08D8-3F48-4E18-98E3-9B53ACB6C6D9}" name="Treatment stage T">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="20" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11259,7 +11268,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="19" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="29" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="D112:G117" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -13300,7 +13309,7 @@
     </row>
     <row r="142" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="39" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E142" s="39" t="s">
         <v>95</v>
@@ -13990,7 +13999,7 @@
         <v>10</v>
       </c>
       <c r="E206" s="39" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="207" spans="4:8" x14ac:dyDescent="0.25">
@@ -14865,7 +14874,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="137" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15120,16 +15129,16 @@
         <v>288</v>
       </c>
       <c r="E13" s="128" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="F13" s="57" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="G13" s="128">
         <v>0</v>
       </c>
       <c r="H13" s="57" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="24"/>
@@ -15145,16 +15154,16 @@
         <v>289</v>
       </c>
       <c r="E14" s="128" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="F14" s="57" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="G14" s="128">
         <v>0</v>
       </c>
       <c r="H14" s="57" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="24"/>
@@ -15200,7 +15209,7 @@
       </c>
       <c r="C17" s="24"/>
       <c r="D17" s="115" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -15217,7 +15226,7 @@
       </c>
       <c r="C18" s="24"/>
       <c r="D18" s="133" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -15249,19 +15258,19 @@
       </c>
       <c r="C20" s="24"/>
       <c r="D20" s="135" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="E20" s="135" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="F20" s="135" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="G20" s="135" t="s">
         <v>319</v>
       </c>
       <c r="H20" s="135" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="24"/>
@@ -15270,7 +15279,7 @@
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="24"/>
       <c r="D21" s="1" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="E21" s="134">
         <f>'4.1.1.9 Manure applied to soils'!$E$56</f>
@@ -15281,10 +15290,10 @@
         <v>kg N</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>322</v>
+        <v>344</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="24"/>
@@ -15293,7 +15302,7 @@
     <row r="22" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="24"/>
       <c r="D22" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E22" s="134">
         <f>'4.1.1.9 Manure applied to soils'!$E$104</f>
@@ -15304,10 +15313,10 @@
         <v>kg N</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="24"/>
@@ -15316,7 +15325,7 @@
     <row r="23" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="24"/>
       <c r="D23" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E23" s="134">
         <f>'4.1.1.9 Manure applied to soils'!$E$123</f>
@@ -15327,10 +15336,10 @@
         <v>kg N</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="I23" s="1"/>
       <c r="J23" s="24"/>
@@ -17016,7 +17025,7 @@
         <v>4.1.1.5-6 Atmospheric deposition</v>
       </c>
       <c r="D13" s="66" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E13" s="41" t="s">
         <v>148</v>
@@ -17131,7 +17140,7 @@
         <v>Constants - Common</v>
       </c>
       <c r="D19" s="66" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E19" s="41" t="s">
         <v>148</v>
@@ -17501,7 +17510,7 @@
     </row>
     <row r="53" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D53" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E53" s="49">
         <v>0.25</v>
@@ -17562,7 +17571,7 @@
     </row>
     <row r="58" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D58" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E58" s="49">
         <v>0.25</v>
@@ -23322,7 +23331,8 @@
     <row r="165" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -26427,7 +26437,7 @@
         <f t="array" ref="H89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.03</v>
       </c>
-      <c r="I89" s="39" t="str" cm="1">
+      <c r="I89" s="138" t="str" cm="1">
         <f t="array" ref="I89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26443,7 +26453,7 @@
         <f t="array" ref="L89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.01</v>
       </c>
-      <c r="M89" s="39" t="str" cm="1">
+      <c r="M89" s="138" t="str" cm="1">
         <f t="array" ref="M89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26473,7 +26483,7 @@
         <f t="array" ref="H90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.02</v>
       </c>
-      <c r="I90" s="39" t="str" cm="1">
+      <c r="I90" s="138" t="str" cm="1">
         <f t="array" ref="I90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26489,7 +26499,7 @@
         <f t="array" ref="L90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.02</v>
       </c>
-      <c r="M90" s="39" t="str" cm="1">
+      <c r="M90" s="138" t="str" cm="1">
         <f t="array" ref="M90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26519,7 +26529,7 @@
         <f t="array" ref="H91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.01</v>
       </c>
-      <c r="I91" s="39" t="str" cm="1">
+      <c r="I91" s="138" t="str" cm="1">
         <f t="array" ref="I91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26535,7 +26545,7 @@
         <f t="array" ref="L91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.01</v>
       </c>
-      <c r="M91" s="39" t="str" cm="1">
+      <c r="M91" s="138" t="str" cm="1">
         <f t="array" ref="M91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26565,7 +26575,7 @@
         <f t="array" ref="H92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0</v>
       </c>
-      <c r="I92" s="39" t="str" cm="1">
+      <c r="I92" s="138" t="str" cm="1">
         <f t="array" ref="I92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26581,7 +26591,7 @@
         <f t="array" ref="L92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0</v>
       </c>
-      <c r="M92" s="39" t="str" cm="1">
+      <c r="M92" s="138" t="str" cm="1">
         <f t="array" ref="M92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26611,7 +26621,7 @@
         <f t="array" ref="H93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.77</v>
       </c>
-      <c r="I93" s="39" t="str" cm="1">
+      <c r="I93" s="138" t="str" cm="1">
         <f t="array" ref="I93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26627,7 +26637,7 @@
         <f t="array" ref="L93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.77</v>
       </c>
-      <c r="M93" s="39" t="str" cm="1">
+      <c r="M93" s="138" t="str" cm="1">
         <f t="array" ref="M93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26637,7 +26647,12 @@
       </c>
     </row>
     <row r="94" spans="4:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M94" s="24"/>
+      <c r="I94" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="M94" s="24" t="s">
+        <v>342</v>
+      </c>
     </row>
     <row r="95" spans="4:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="M95" s="24"/>

</xml_diff>

<commit_message>
add swine mms, partial poultry mms
</commit_message>
<xml_diff>
--- a/Excel/4_1_ManureManagement_Feedlot_WIP_v04.xlsx
+++ b/Excel/4_1_ManureManagement_Feedlot_WIP_v04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C629B843-A630-4B85-8DD5-D8E2F16401AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFD461C-6A40-4AFC-8798-512CF117937D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" firstSheet="9" activeTab="9" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1080" yWindow="690" windowWidth="36585" windowHeight="19950" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -27,9 +27,6 @@
     <sheet name="Acknowledgements" sheetId="72" r:id="rId12"/>
     <sheet name="Tab template" sheetId="74" r:id="rId13"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId14"/>
-  </externalReferences>
   <definedNames>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -479,7 +476,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="338">
   <si>
     <t>Home</t>
   </si>
@@ -1464,50 +1461,7 @@
     <t>Mass of N applied to soils (Method 1)</t>
   </si>
   <si>
-    <t>Table_PF_sold</t>
-  </si>
-  <si>
-    <t>Fraction of manure sold</t>
-  </si>
-  <si>
-    <t>M1_Table_MNSoil_scope3_sold</t>
-  </si>
-  <si>
-    <t>M2_Table_MNSoil_scope3_sold</t>
-  </si>
-  <si>
-    <t>Mass of N sold as fertiliser (Method 2)</t>
-  </si>
-  <si>
-    <t>Mass of N sold as fertiliser (Method 1)</t>
-  </si>
-  <si>
-    <t>Mass of nitrogen applied as fertiliser on own farm</t>
-  </si>
-  <si>
-    <t>Mass of nitrogen sold</t>
-  </si>
-  <si>
-    <r>
-      <t>MNSoil</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <vertAlign val="subscript"/>
-        <sz val="16"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>scope3,sold</t>
-    </r>
-  </si>
-  <si>
     <t>* Manure that is removed from stage 2 and 3 MMS and used as fertiliser on the farm, for other enterprises (eg crops)</t>
-  </si>
-  <si>
-    <t>* Manure that is removed from stage 2 and 3 MMS that is sold</t>
   </si>
   <si>
     <r>
@@ -1599,9 +1553,6 @@
     </r>
   </si>
   <si>
-    <t>Where deposited on farm soils as waste, what is the closest match?</t>
-  </si>
-  <si>
     <t>lacking subscripts</t>
   </si>
   <si>
@@ -1717,9 +1668,6 @@
     <t>Method 2 custom values (Edit if known)</t>
   </si>
   <si>
-    <t>Applied to farm soils as fertiliser</t>
-  </si>
-  <si>
     <t>Irrigation type i</t>
   </si>
   <si>
@@ -1735,9 +1683,6 @@
     <t>use vic</t>
   </si>
   <si>
-    <t>Manure nitrogen deposited on farm soils (excluding farm fertiliser use)</t>
-  </si>
-  <si>
     <t>Scope 1 - This feedlot</t>
   </si>
   <si>
@@ -1748,6 +1693,15 @@
   </si>
   <si>
     <t>Acknowledgements</t>
+  </si>
+  <si>
+    <t>Where manure was deposited on farm soils, what is the closest match?</t>
+  </si>
+  <si>
+    <t>Scope 1: Mass of nitrogen applied as fertiliser on own farm</t>
+  </si>
+  <si>
+    <t>Manure nitrogen deposited on farm soils (including use as fertiliser for other enterprises on own farm eg crops)</t>
   </si>
 </sst>
 </file>
@@ -2285,7 +2239,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -2515,24 +2469,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="3" tint="0.749961851863155"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="3" tint="0.749961851863155"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2713,7 +2649,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="40" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -3053,16 +2989,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="13" borderId="0" xfId="41" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="47" fillId="13" borderId="10" xfId="41" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="13" borderId="21" xfId="41" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="13" borderId="22" xfId="41" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -3169,486 +3096,6 @@
     <cellStyle name="Unit total" xfId="26" xr:uid="{65428923-3DAD-47B6-8DDF-0EBD05E7C55B}"/>
   </cellStyles>
   <dxfs count="60">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -4224,6 +3671,486 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
@@ -10692,26 +10619,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Home"/>
-      <sheetName val="Constants - Common"/>
-      <sheetName val="Acknowledgements"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -10795,34 +10702,34 @@
     <tableColumn id="1" xr3:uid="{3885FE93-299E-44EB-B503-99C305BD6F41}" name="Treatment stage T">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D0E12F95-AC29-47D0-913A-0A0B02931616}" name="MMS m" dataDxfId="47" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{D0E12F95-AC29-47D0-913A-0A0B02931616}" name="MMS m" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E17BE7AB-8FAD-4B5C-9F86-E70E6A00B9B1}" name="NSW" dataDxfId="46" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{E17BE7AB-8FAD-4B5C-9F86-E70E6A00B9B1}" name="NSW" dataDxfId="26" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D4C6F922-2719-4479-B7CC-26C5286F73ED}" name="ACT" dataDxfId="45" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{D4C6F922-2719-4479-B7CC-26C5286F73ED}" name="ACT" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5034DCA1-F046-43BC-A94F-832832E6D634}" name="QLD" dataDxfId="44" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5034DCA1-F046-43BC-A94F-832832E6D634}" name="QLD" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="43" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="21" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="40" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="20" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="39" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="38" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -10938,49 +10845,49 @@
     <tableColumn id="1" xr3:uid="{62AAF798-B15D-4271-927A-A8A3761FCCCC}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8717C2F5-373F-46C4-9931-0F5D03C661C8}" name="MAT" totalsRowDxfId="19" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{8717C2F5-373F-46C4-9931-0F5D03C661C8}" name="MAT" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{C4680CAC-71CD-41BE-8D7D-8DA3A191C6AD}" name="MAP" totalsRowDxfId="18" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{C4680CAC-71CD-41BE-8D7D-8DA3A191C6AD}" name="MAP" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D4E26F30-4195-4CE8-B4DA-99F110B90518}" name="Frost days per year" totalsRowDxfId="17" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{D4E26F30-4195-4CE8-B4DA-99F110B90518}" name="Frost days per year" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0DF39DDE-3EFC-4342-A2A9-4182097B7EC1}" name="Elevation" totalsRowDxfId="16" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{0DF39DDE-3EFC-4342-A2A9-4182097B7EC1}" name="Elevation" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{3A9CEA3D-76B5-41DC-82F7-4841CE23DEC7}" name="MAP:PET" totalsRowDxfId="15" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{3A9CEA3D-76B5-41DC-82F7-4841CE23DEC7}" name="MAP:PET" totalsRowDxfId="43" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{BC2DED34-2933-4483-B3FF-07D5615064C6}" name="Min temp" totalsRowDxfId="14" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{BC2DED34-2933-4483-B3FF-07D5615064C6}" name="Min temp" totalsRowDxfId="42" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{FF01D565-BF4F-4999-BD32-018FB684F25C}" name="Max temp" totalsRowDxfId="13" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{FF01D565-BF4F-4999-BD32-018FB684F25C}" name="Max temp" totalsRowDxfId="41" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{7CF1165F-54EC-4690-A7F1-470C0A20CC1D}" name="Min rainfall" totalsRowDxfId="12" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{7CF1165F-54EC-4690-A7F1-470C0A20CC1D}" name="Min rainfall" totalsRowDxfId="40" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{AED5C66B-6ACD-48DC-8C8B-05C15217CA0B}" name="Max rainfall" totalsRowDxfId="11" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{AED5C66B-6ACD-48DC-8C8B-05C15217CA0B}" name="Max rainfall" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{E41B7A22-BEF4-46C0-8A2D-2792B8AF3565}" name="Min frost days" totalsRowDxfId="10" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{E41B7A22-BEF4-46C0-8A2D-2792B8AF3565}" name="Min frost days" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{2027D86C-E675-4004-BA7D-52312C234326}" name="Max frost days" totalsRowDxfId="9" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{2027D86C-E675-4004-BA7D-52312C234326}" name="Max frost days" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{5CE42D6C-D9F0-43B0-A4CE-78C7DA6F0FF8}" name="Min elevation" totalsRowDxfId="8" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{5CE42D6C-D9F0-43B0-A4CE-78C7DA6F0FF8}" name="Min elevation" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{2847C6FC-AAAB-4377-9BB4-0CE7770C5FCD}" name="Max elevation" totalsRowDxfId="7" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{2847C6FC-AAAB-4377-9BB4-0CE7770C5FCD}" name="Max elevation" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{A1A7A932-493E-40FC-9996-02E450D40A76}" name="Min MAP:PET" totalsRowDxfId="6" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{A1A7A932-493E-40FC-9996-02E450D40A76}" name="Min MAP:PET" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{578E0E27-B0A1-4C90-AC88-4F16A7913682}" name="Max MAP:PET" totalsRowDxfId="5" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{578E0E27-B0A1-4C90-AC88-4F16A7913682}" name="Max MAP:PET" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -10998,7 +10905,7 @@
     <tableColumn id="1" xr3:uid="{DE69BEA7-39B3-406C-A179-3B18221DDF1E}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{189B94EF-4D9E-415D-AE6B-6B0CA1291C92}" name="Wet or Dry Zone" totalsRowDxfId="4" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{189B94EF-4D9E-415D-AE6B-6B0CA1291C92}" name="Wet or Dry Zone" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11102,7 +11009,7 @@
   </autoFilter>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{F2B173A3-CADE-4DCA-988D-39EE2392D8DB}" name="MMS"/>
-    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="37" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="17" dataCellStyle="Content normal"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11118,7 +11025,7 @@
     <tableColumn id="1" xr3:uid="{3955BCED-58D4-4A02-A1B0-5CC59B870E09}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{96C4C42E-00DA-40A3-82DD-B42796163C14}" name="FracWET" dataDxfId="3">
+    <tableColumn id="2" xr3:uid="{96C4C42E-00DA-40A3-82DD-B42796163C14}" name="FracWET" dataDxfId="31">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11166,7 +11073,7 @@
     <tableColumn id="1" xr3:uid="{21644B2F-35C5-46C7-9C1B-01B9C9438466}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{44113FA0-3C8F-47F8-BEAF-F6E5E8D642A7}" name="FracWET" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{44113FA0-3C8F-47F8-BEAF-F6E5E8D642A7}" name="FracWET" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11184,7 +11091,7 @@
     <tableColumn id="1" xr3:uid="{E0DC9C67-4A93-426B-B45D-29C1739DBF9F}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5B0E4755-347F-4448-8061-D1B2ADD5FCE9}" name="EFPRP" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{5B0E4755-347F-4448-8061-D1B2ADD5FCE9}" name="EFPRP" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11202,7 +11109,7 @@
     <tableColumn id="1" xr3:uid="{1B40AF4E-D0D3-47D2-8A92-B9C2CADD3D81}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{60B3218D-7B8C-4E84-A9EC-F5BEE02E1FC4}" name="Season" dataDxfId="0" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{60B3218D-7B8C-4E84-A9EC-F5BEE02E1FC4}" name="Season" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11247,22 +11154,22 @@
     <tableColumn id="1" xr3:uid="{FDCB848C-205F-48EA-BACF-F54BCD324E05}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="36" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="33" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="32" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11285,22 +11192,22 @@
     <tableColumn id="1" xr3:uid="{96F6B4E3-E1EE-445F-9BCE-628B89FC3727}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="28" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="25" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11318,7 +11225,7 @@
     <tableColumn id="1" xr3:uid="{9D472457-4D8B-44ED-9567-B889D058C2F1}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="24" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="4" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11338,13 +11245,13 @@
     <tableColumn id="1" xr3:uid="{C80C08D8-3F48-4E18-98E3-9B53ACB6C6D9}" name="Treatment stage T">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="23" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="3" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="2" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="1" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11353,7 +11260,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="20" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="0" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="D112:G117" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -13400,7 +13307,7 @@
     </row>
     <row r="142" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="39" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="E142" s="39" t="s">
         <v>95</v>
@@ -13760,16 +13667,16 @@
     </row>
     <row r="186" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D186" s="39" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="E186" s="39" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="F186" s="39" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="G186" s="39" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="H186" s="39" t="s">
         <v>36</v>
@@ -14090,7 +13997,7 @@
         <v>10</v>
       </c>
       <c r="E206" s="39" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
     </row>
     <row r="207" spans="4:8" x14ac:dyDescent="0.25">
@@ -14121,10 +14028,10 @@
     </row>
     <row r="212" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D212" s="39" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
       <c r="E212" s="39" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
     </row>
     <row r="213" spans="4:5" x14ac:dyDescent="0.25">
@@ -14697,7 +14604,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -15091,7 +14998,7 @@
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
     <col min="2" max="3" width="2.7109375" customWidth="1"/>
-    <col min="4" max="4" width="78.42578125" customWidth="1"/>
+    <col min="4" max="4" width="96.28515625" customWidth="1"/>
     <col min="5" max="6" width="28.7109375" customWidth="1"/>
     <col min="7" max="7" width="40.28515625" customWidth="1"/>
     <col min="8" max="8" width="59.7109375" customWidth="1"/>
@@ -15105,8 +15012,8 @@
       <c r="A1" s="71" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C1" s="137" t="s">
-        <v>334</v>
+      <c r="C1" s="134" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15129,7 +15036,7 @@
       <c r="K3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="136" t="str">
+      <c r="A4" s="133" t="str">
         <f>HYPERLINK("#'Results'!A1", "Results")</f>
         <v>Results</v>
       </c>
@@ -15162,20 +15069,20 @@
         <v>3</v>
       </c>
       <c r="C6" s="24"/>
-      <c r="D6" s="135" t="s">
-        <v>292</v>
-      </c>
-      <c r="E6" s="135" t="s">
-        <v>290</v>
-      </c>
-      <c r="F6" s="135" t="s">
-        <v>320</v>
-      </c>
-      <c r="G6" s="135" t="s">
-        <v>291</v>
-      </c>
-      <c r="H6" s="135" t="s">
-        <v>321</v>
+      <c r="D6" s="132" t="s">
+        <v>282</v>
+      </c>
+      <c r="E6" s="132" t="s">
+        <v>280</v>
+      </c>
+      <c r="F6" s="132" t="s">
+        <v>309</v>
+      </c>
+      <c r="G6" s="132" t="s">
+        <v>281</v>
+      </c>
+      <c r="H6" s="132" t="s">
+        <v>310</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="24"/>
@@ -15188,9 +15095,9 @@
       </c>
       <c r="C7" s="24"/>
       <c r="D7" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="E7" s="128">
+        <v>272</v>
+      </c>
+      <c r="E7" s="125">
         <f>'4.1.1.1-2 Methane'!E164</f>
         <v>2.7938769470975995</v>
       </c>
@@ -15198,7 +15105,7 @@
         <f>'4.1.1.1-2 Methane'!F164</f>
         <v>t CH4</v>
       </c>
-      <c r="G7" s="128">
+      <c r="G7" s="125">
         <f>'4.1.1.1-2 Methane'!E169</f>
         <v>78.228554518732778</v>
       </c>
@@ -15217,9 +15124,9 @@
       </c>
       <c r="C8" s="24"/>
       <c r="D8" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="E8" s="128">
+        <v>273</v>
+      </c>
+      <c r="E8" s="125">
         <f>'4.1.1.1-2 Methane'!N164</f>
         <v>2.7938769470975995</v>
       </c>
@@ -15227,7 +15134,7 @@
         <f>'4.1.1.1-2 Methane'!O164</f>
         <v>t CH4</v>
       </c>
-      <c r="G8" s="128">
+      <c r="G8" s="125">
         <f>'4.1.1.1-2 Methane'!N169</f>
         <v>78.228554518732778</v>
       </c>
@@ -15243,9 +15150,9 @@
       <c r="A9" s="17"/>
       <c r="C9" s="24"/>
       <c r="D9" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="E9" s="128">
+        <v>274</v>
+      </c>
+      <c r="E9" s="125">
         <f>'4.1.1.3-4 Direct N20'!E207</f>
         <v>1.0745527700847912</v>
       </c>
@@ -15253,7 +15160,7 @@
         <f>'4.1.1.3-4 Direct N20'!F207</f>
         <v>t N2O</v>
       </c>
-      <c r="G9" s="128">
+      <c r="G9" s="125">
         <f>'4.1.1.3-4 Direct N20'!E212</f>
         <v>284.75648407246968</v>
       </c>
@@ -15271,9 +15178,9 @@
       </c>
       <c r="C10" s="24"/>
       <c r="D10" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="E10" s="128">
+        <v>275</v>
+      </c>
+      <c r="E10" s="125">
         <f>'4.1.1.3-4 Direct N20'!M207</f>
         <v>1.0745527700847912</v>
       </c>
@@ -15281,7 +15188,7 @@
         <f>'4.1.1.3-4 Direct N20'!N207</f>
         <v>t N2O</v>
       </c>
-      <c r="G10" s="128">
+      <c r="G10" s="125">
         <f>'4.1.1.3-4 Direct N20'!M212</f>
         <v>284.75648407246968</v>
       </c>
@@ -15300,9 +15207,9 @@
       </c>
       <c r="C11" s="24"/>
       <c r="D11" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="E11" s="128">
+        <v>276</v>
+      </c>
+      <c r="E11" s="125">
         <f>'4.1.1.5-6 Atmos Deposition'!$E$60</f>
         <v>0.16441385070403455</v>
       </c>
@@ -15310,7 +15217,7 @@
         <f>'4.1.1.5-6 Atmos Deposition'!$F$60</f>
         <v>t N2O</v>
       </c>
-      <c r="G11" s="128">
+      <c r="G11" s="125">
         <f>'4.1.1.5-6 Atmos Deposition'!$E$65</f>
         <v>43.569670436569155</v>
       </c>
@@ -15329,9 +15236,9 @@
       </c>
       <c r="C12" s="24"/>
       <c r="D12" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="E12" s="128">
+        <v>277</v>
+      </c>
+      <c r="E12" s="125">
         <f>'4.1.1.5-6 Atmos Deposition'!$M$60</f>
         <v>0.16441385070403455</v>
       </c>
@@ -15339,7 +15246,7 @@
         <f>'4.1.1.5-6 Atmos Deposition'!$N$60</f>
         <v>t N2O</v>
       </c>
-      <c r="G12" s="128">
+      <c r="G12" s="125">
         <f>'4.1.1.5-6 Atmos Deposition'!$M$65</f>
         <v>43.569670436569155</v>
       </c>
@@ -15358,19 +15265,19 @@
       </c>
       <c r="C13" s="24"/>
       <c r="D13" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="E13" s="128" t="s">
-        <v>333</v>
+        <v>278</v>
+      </c>
+      <c r="E13" s="125" t="s">
+        <v>322</v>
       </c>
       <c r="F13" s="57" t="s">
-        <v>333</v>
-      </c>
-      <c r="G13" s="128">
+        <v>322</v>
+      </c>
+      <c r="G13" s="125">
         <v>0</v>
       </c>
       <c r="H13" s="57" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="24"/>
@@ -15383,19 +15290,19 @@
       </c>
       <c r="C14" s="24"/>
       <c r="D14" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="E14" s="128" t="s">
-        <v>333</v>
+        <v>279</v>
+      </c>
+      <c r="E14" s="125" t="s">
+        <v>322</v>
       </c>
       <c r="F14" s="57" t="s">
-        <v>333</v>
-      </c>
-      <c r="G14" s="128">
+        <v>322</v>
+      </c>
+      <c r="G14" s="125">
         <v>0</v>
       </c>
       <c r="H14" s="57" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="24"/>
@@ -15404,11 +15311,11 @@
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="24"/>
       <c r="D15" s="31" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="E15" s="25"/>
       <c r="F15" s="31"/>
-      <c r="G15" s="132">
+      <c r="G15" s="129">
         <f>SUM(G7:G14)</f>
         <v>813.10941805554319</v>
       </c>
@@ -15441,7 +15348,7 @@
       </c>
       <c r="C17" s="24"/>
       <c r="D17" s="115" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -15457,8 +15364,8 @@
         <v>Constants - Livestock</v>
       </c>
       <c r="C18" s="24"/>
-      <c r="D18" s="133" t="s">
-        <v>332</v>
+      <c r="D18" s="130" t="s">
+        <v>321</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -15489,20 +15396,20 @@
         <v>Acknowledgements</v>
       </c>
       <c r="C20" s="24"/>
-      <c r="D20" s="135" t="s">
-        <v>327</v>
-      </c>
-      <c r="E20" s="135" t="s">
-        <v>324</v>
-      </c>
-      <c r="F20" s="135" t="s">
-        <v>325</v>
-      </c>
-      <c r="G20" s="135" t="s">
-        <v>319</v>
-      </c>
-      <c r="H20" s="135" t="s">
-        <v>331</v>
+      <c r="D20" s="132" t="s">
+        <v>316</v>
+      </c>
+      <c r="E20" s="132" t="s">
+        <v>313</v>
+      </c>
+      <c r="F20" s="132" t="s">
+        <v>314</v>
+      </c>
+      <c r="G20" s="132" t="s">
+        <v>308</v>
+      </c>
+      <c r="H20" s="132" t="s">
+        <v>320</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="24"/>
@@ -15511,21 +15418,21 @@
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="24"/>
       <c r="D21" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="E21" s="134">
+        <v>337</v>
+      </c>
+      <c r="E21" s="131">
         <f>'4.1.1.9 Manure applied to soils'!$E$56</f>
-        <v>9574.3563485022751</v>
+        <v>14361.534522753413</v>
       </c>
       <c r="F21" s="57" t="str">
         <f>'4.1.1.9 Manure applied to soils'!$F$56</f>
         <v>kg N</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="24"/>
@@ -15534,21 +15441,21 @@
     <row r="22" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="24"/>
       <c r="D22" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="E22" s="134">
-        <f>'4.1.1.9 Manure applied to soils'!$E$104</f>
+        <v>317</v>
+      </c>
+      <c r="E22" s="131">
+        <f>'4.1.1.9 Manure applied to soils'!$E$103</f>
         <v>4787.1781742511375</v>
       </c>
       <c r="F22" s="57" t="str">
-        <f>'4.1.1.9 Manure applied to soils'!$F$104</f>
+        <f>'4.1.1.9 Manure applied to soils'!$F$103</f>
         <v>kg N</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="24"/>
@@ -15557,21 +15464,21 @@
     <row r="23" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="24"/>
       <c r="D23" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="E23" s="134">
-        <f>'4.1.1.9 Manure applied to soils'!$E$123</f>
+        <v>311</v>
+      </c>
+      <c r="E23" s="131">
+        <f>'4.1.1.9 Manure applied to soils'!E81</f>
         <v>4787.1781742511375</v>
       </c>
       <c r="F23" s="57" t="str">
-        <f>'4.1.1.9 Manure applied to soils'!$F$123</f>
+        <f>'4.1.1.9 Manure applied to soils'!F81</f>
         <v>kg N</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="I23" s="1"/>
       <c r="J23" s="24"/>
@@ -15738,8 +15645,8 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
-      <c r="I38" s="127"/>
-      <c r="J38" s="127"/>
+      <c r="I38" s="124"/>
+      <c r="J38" s="124"/>
       <c r="K38" s="24"/>
     </row>
     <row r="39" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15749,8 +15656,8 @@
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
-      <c r="I39" s="127"/>
-      <c r="J39" s="127"/>
+      <c r="I39" s="124"/>
+      <c r="J39" s="124"/>
       <c r="K39" s="24"/>
     </row>
     <row r="40" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15760,8 +15667,8 @@
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
-      <c r="I40" s="127"/>
-      <c r="J40" s="127"/>
+      <c r="I40" s="124"/>
+      <c r="J40" s="124"/>
       <c r="K40" s="24"/>
     </row>
     <row r="41" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15771,8 +15678,8 @@
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
-      <c r="I41" s="127"/>
-      <c r="J41" s="127"/>
+      <c r="I41" s="124"/>
+      <c r="J41" s="124"/>
       <c r="K41" s="24"/>
     </row>
     <row r="42" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15782,8 +15689,8 @@
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
-      <c r="I42" s="127"/>
-      <c r="J42" s="127"/>
+      <c r="I42" s="124"/>
+      <c r="J42" s="124"/>
       <c r="K42" s="24"/>
     </row>
     <row r="43" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15793,8 +15700,8 @@
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
-      <c r="I43" s="127"/>
-      <c r="J43" s="127"/>
+      <c r="I43" s="124"/>
+      <c r="J43" s="124"/>
       <c r="K43" s="24"/>
     </row>
     <row r="44" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15804,8 +15711,8 @@
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
-      <c r="I44" s="127"/>
-      <c r="J44" s="127"/>
+      <c r="I44" s="124"/>
+      <c r="J44" s="124"/>
       <c r="K44" s="24"/>
     </row>
     <row r="45" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15815,8 +15722,8 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
-      <c r="I45" s="127"/>
-      <c r="J45" s="127"/>
+      <c r="I45" s="124"/>
+      <c r="J45" s="124"/>
       <c r="K45" s="24"/>
     </row>
     <row r="46" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15826,8 +15733,8 @@
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
-      <c r="I46" s="127"/>
-      <c r="J46" s="127"/>
+      <c r="I46" s="124"/>
+      <c r="J46" s="124"/>
       <c r="K46" s="24"/>
     </row>
     <row r="47" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15837,8 +15744,8 @@
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
-      <c r="I47" s="127"/>
-      <c r="J47" s="127"/>
+      <c r="I47" s="124"/>
+      <c r="J47" s="124"/>
       <c r="K47" s="24"/>
     </row>
     <row r="48" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15848,8 +15755,8 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
-      <c r="I48" s="127"/>
-      <c r="J48" s="127"/>
+      <c r="I48" s="124"/>
+      <c r="J48" s="124"/>
       <c r="K48" s="24"/>
     </row>
     <row r="49" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15858,9 +15765,9 @@
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
-      <c r="H49" s="127"/>
-      <c r="I49" s="127"/>
-      <c r="J49" s="127"/>
+      <c r="H49" s="124"/>
+      <c r="I49" s="124"/>
+      <c r="J49" s="124"/>
       <c r="K49" s="24"/>
     </row>
     <row r="50" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15869,9 +15776,9 @@
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
-      <c r="H50" s="127"/>
-      <c r="I50" s="127"/>
-      <c r="J50" s="127"/>
+      <c r="H50" s="124"/>
+      <c r="I50" s="124"/>
+      <c r="J50" s="124"/>
       <c r="K50" s="24"/>
     </row>
     <row r="51" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15880,9 +15787,9 @@
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
-      <c r="H51" s="127"/>
-      <c r="I51" s="127"/>
-      <c r="J51" s="127"/>
+      <c r="H51" s="124"/>
+      <c r="I51" s="124"/>
+      <c r="J51" s="124"/>
       <c r="K51" s="24"/>
     </row>
     <row r="52" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15891,9 +15798,9 @@
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
-      <c r="H52" s="127"/>
-      <c r="I52" s="127"/>
-      <c r="J52" s="127"/>
+      <c r="H52" s="124"/>
+      <c r="I52" s="124"/>
+      <c r="J52" s="124"/>
       <c r="K52" s="24"/>
     </row>
     <row r="53" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15902,9 +15809,9 @@
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
-      <c r="H53" s="127"/>
-      <c r="I53" s="127"/>
-      <c r="J53" s="127"/>
+      <c r="H53" s="124"/>
+      <c r="I53" s="124"/>
+      <c r="J53" s="124"/>
       <c r="K53" s="24"/>
     </row>
     <row r="54" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -17257,7 +17164,7 @@
         <v>4.1.1.5-6 Atmospheric deposition</v>
       </c>
       <c r="D13" s="66" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="E13" s="41" t="s">
         <v>148</v>
@@ -17372,7 +17279,7 @@
         <v>Constants - Common</v>
       </c>
       <c r="D19" s="66" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="E19" s="41" t="s">
         <v>148</v>
@@ -17681,7 +17588,7 @@
     </row>
     <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D48" s="1" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="E48" s="49">
         <v>0.25</v>
@@ -17742,7 +17649,7 @@
     </row>
     <row r="53" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D53" s="1" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="E53" s="49">
         <v>0.25</v>
@@ -17803,7 +17710,7 @@
     </row>
     <row r="58" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D58" s="1" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="E58" s="49">
         <v>0.25</v>
@@ -17844,10 +17751,10 @@
     <row r="61" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="62" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D62" s="1" t="s">
-        <v>302</v>
+        <v>335</v>
       </c>
       <c r="E62" s="42" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>11</v>
@@ -17855,7 +17762,7 @@
     </row>
     <row r="63" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E63" s="42" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>11</v>
@@ -18023,7 +17930,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2" spans="1:19" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -20178,7 +20085,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -22483,7 +22390,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -22634,10 +22541,10 @@
         <v>Constants - Feedlot</v>
       </c>
       <c r="D17" s="105" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="L17" s="105" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -22646,10 +22553,10 @@
         <v>Constants - Livestock</v>
       </c>
       <c r="D18" s="104" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="L18" s="104" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -22920,18 +22827,18 @@
     <row r="32" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D33" s="105" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="L33" s="105" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
     </row>
     <row r="34" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D34" s="104" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="L34" s="104" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
     </row>
     <row r="35" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -23126,45 +23033,45 @@
     </row>
     <row r="40" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D41" s="131" t="s">
-        <v>301</v>
+      <c r="D41" s="128" t="s">
+        <v>291</v>
       </c>
       <c r="E41" s="48">
         <f>SUM(E36:G39)</f>
         <v>58126.108834759696</v>
       </c>
-      <c r="F41" s="129" t="str">
+      <c r="F41" s="126" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
-      <c r="L41" s="131" t="s">
-        <v>301</v>
+      <c r="L41" s="128" t="s">
+        <v>291</v>
       </c>
       <c r="M41" s="48">
         <f>SUM(M36:O39)</f>
         <v>58126.108834759696</v>
       </c>
-      <c r="N41" s="129" t="str">
+      <c r="N41" s="126" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
     </row>
     <row r="42" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="43" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C43" s="130"/>
-      <c r="D43" s="130"/>
-      <c r="E43" s="130"/>
-      <c r="F43" s="130"/>
-      <c r="G43" s="130"/>
-      <c r="H43" s="130"/>
-      <c r="I43" s="130"/>
-      <c r="K43" s="130"/>
-      <c r="L43" s="130"/>
-      <c r="M43" s="130"/>
-      <c r="N43" s="130"/>
-      <c r="O43" s="130"/>
-      <c r="P43" s="130"/>
-      <c r="Q43" s="130"/>
+      <c r="C43" s="127"/>
+      <c r="D43" s="127"/>
+      <c r="E43" s="127"/>
+      <c r="F43" s="127"/>
+      <c r="G43" s="127"/>
+      <c r="H43" s="127"/>
+      <c r="I43" s="127"/>
+      <c r="K43" s="127"/>
+      <c r="L43" s="127"/>
+      <c r="M43" s="127"/>
+      <c r="N43" s="127"/>
+      <c r="O43" s="127"/>
+      <c r="P43" s="127"/>
+      <c r="Q43" s="127"/>
     </row>
     <row r="44" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="45" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -23250,7 +23157,7 @@
         <v>1.8E-3</v>
       </c>
       <c r="H54" s="117" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="L54" s="60" t="str">
         <v>EF_N2O</v>
@@ -23363,7 +23270,7 @@
     <row r="59" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="60" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D60" s="110" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="E60" s="111" cm="1">
         <f t="array" ref="E60">MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions(G53,G54,G55)</f>
@@ -23374,7 +23281,7 @@
         <v>t N2O</v>
       </c>
       <c r="L60" s="110" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="M60" s="111" cm="1">
         <f t="array" ref="M60">MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions(O53,O54,O55)</f>
@@ -24116,16 +24023,16 @@
         <v>Solid storage</v>
       </c>
       <c r="E45" s="55">
-        <f>'Input - Feedlot'!E49</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!E48+'Input - Feedlot'!E49</f>
+        <v>0.75</v>
       </c>
       <c r="F45" s="55">
-        <f>'Input - Feedlot'!F49</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!F48+'Input - Feedlot'!F49</f>
+        <v>0.75</v>
       </c>
       <c r="G45" s="55">
-        <f>'Input - Feedlot'!G49</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!G48+'Input - Feedlot'!G49</f>
+        <v>0.75</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>101</v>
@@ -24137,16 +24044,16 @@
         <v>Composting (passive windrow)</v>
       </c>
       <c r="E46" s="55">
-        <f>'Input - Feedlot'!E54</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!E53+'Input - Feedlot'!E54</f>
+        <v>0.75</v>
       </c>
       <c r="F46" s="55">
-        <f>'Input - Feedlot'!F54</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!F53+'Input - Feedlot'!F54</f>
+        <v>0.75</v>
       </c>
       <c r="G46" s="55">
-        <f>'Input - Feedlot'!G54</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!G53+'Input - Feedlot'!G54</f>
+        <v>0.75</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>101</v>
@@ -24158,16 +24065,16 @@
         <v>Anaerobic lagoon</v>
       </c>
       <c r="E47" s="55">
-        <f>'Input - Feedlot'!E59</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!E58+'Input - Feedlot'!E59</f>
+        <v>0.75</v>
       </c>
       <c r="F47" s="55">
-        <f>'Input - Feedlot'!F59</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!F58+'Input - Feedlot'!F59</f>
+        <v>0.75</v>
       </c>
       <c r="G47" s="55">
-        <f>'Input - Feedlot'!G59</f>
-        <v>0.5</v>
+        <f>'Input - Feedlot'!G58+'Input - Feedlot'!G59</f>
+        <v>0.75</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>101</v>
@@ -24223,15 +24130,15 @@
       </c>
       <c r="E52" s="55" cm="1">
         <f t="array" ref="E52">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E22,$E$30,$E$38,E45)</f>
-        <v>2002.762431581185</v>
+        <v>3004.1436473717777</v>
       </c>
       <c r="F52" s="55" cm="1">
         <f t="array" ref="F52">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F22,$E$30,$E$38,F45)</f>
-        <v>70.727988893184005</v>
+        <v>106.09198333977601</v>
       </c>
       <c r="G52" s="55" cm="1">
         <f t="array" ref="G52">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G22,$E$30,$E$38,G45)</f>
-        <v>102.15557769599998</v>
+        <v>153.23336654399998</v>
       </c>
       <c r="H52" s="2" t="str">
         <f>$E$12</f>
@@ -24243,15 +24150,15 @@
       </c>
       <c r="M52" s="55" cm="1">
         <f t="array" ref="M52">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M22,$E$30,$E$38,E45)</f>
-        <v>2002.762431581185</v>
+        <v>3004.1436473717777</v>
       </c>
       <c r="N52" s="55" cm="1">
         <f t="array" ref="N52">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N22,$E$30,$E$38,F45)</f>
-        <v>70.727988893184005</v>
+        <v>106.09198333977601</v>
       </c>
       <c r="O52" s="55" cm="1">
         <f t="array" ref="O52">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O22,$E$30,$E$38,G45)</f>
-        <v>102.15557769599998</v>
+        <v>153.23336654399998</v>
       </c>
       <c r="P52" s="2" t="str">
         <f>$E$12</f>
@@ -24265,15 +24172,15 @@
       </c>
       <c r="E53" s="55" cm="1">
         <f t="array" ref="E53">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E23,$E$31,$E$39,E46)</f>
-        <v>6344.3212597739548</v>
+        <v>9516.4818896609322</v>
       </c>
       <c r="F53" s="55" cm="1">
         <f t="array" ref="F53">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F23,$E$31,$E$39,F46)</f>
-        <v>224.051078909952</v>
+        <v>336.07661836492798</v>
       </c>
       <c r="G53" s="55" cm="1">
         <f t="array" ref="G53">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G23,$E$31,$E$39,G46)</f>
-        <v>323.60693068799992</v>
+        <v>485.41039603199988</v>
       </c>
       <c r="H53" s="2" t="str">
         <f>$E$12</f>
@@ -24285,15 +24192,15 @@
       </c>
       <c r="M53" s="55" cm="1">
         <f t="array" ref="M53">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M23,$E$31,$E$39,E46)</f>
-        <v>6344.3212597739548</v>
+        <v>9516.4818896609322</v>
       </c>
       <c r="N53" s="55" cm="1">
         <f t="array" ref="N53">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N23,$E$31,$E$39,F46)</f>
-        <v>224.051078909952</v>
+        <v>336.07661836492798</v>
       </c>
       <c r="O53" s="55" cm="1">
         <f t="array" ref="O53">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O23,$E$31,$E$39,G46)</f>
-        <v>323.60693068799992</v>
+        <v>485.41039603199988</v>
       </c>
       <c r="P53" s="2" t="str">
         <f>$E$12</f>
@@ -24307,15 +24214,15 @@
       </c>
       <c r="E54" s="55" cm="1">
         <f t="array" ref="E54">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E24,$E$32,$E$40,E47)</f>
-        <v>466.46466048000019</v>
+        <v>699.69699072000026</v>
       </c>
       <c r="F54" s="55" cm="1">
         <f t="array" ref="F54">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F24,$E$32,$E$40,F47)</f>
-        <v>16.473300480000002</v>
+        <v>24.709950720000002</v>
       </c>
       <c r="G54" s="55" cm="1">
         <f t="array" ref="G54">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G24,$E$32,$E$40,G47)</f>
-        <v>23.793119999999995</v>
+        <v>35.689679999999996</v>
       </c>
       <c r="H54" s="2" t="str">
         <f>$E$12</f>
@@ -24327,15 +24234,15 @@
       </c>
       <c r="M54" s="55" cm="1">
         <f t="array" ref="M54">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M24,$E$32,$E$40,E47)</f>
-        <v>466.46466048000019</v>
+        <v>699.69699072000026</v>
       </c>
       <c r="N54" s="55" cm="1">
         <f t="array" ref="N54">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N24,$E$32,$E$40,F47)</f>
-        <v>16.473300480000002</v>
+        <v>24.709950720000002</v>
       </c>
       <c r="O54" s="55" cm="1">
         <f t="array" ref="O54">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O24,$E$32,$E$40,G47)</f>
-        <v>23.793119999999995</v>
+        <v>35.689679999999996</v>
       </c>
       <c r="P54" s="2" t="str">
         <f>$E$12</f>
@@ -24349,7 +24256,7 @@
       </c>
       <c r="E56" s="111">
         <f>SUM(E52:G54)</f>
-        <v>9574.3563485022751</v>
+        <v>14361.534522753413</v>
       </c>
       <c r="F56" s="112" t="str">
         <f>$E$12</f>
@@ -24360,7 +24267,7 @@
       </c>
       <c r="M56" s="111">
         <f>SUM(M52:O54)</f>
-        <v>9574.3563485022751</v>
+        <v>14361.534522753413</v>
       </c>
       <c r="N56" s="112" t="str">
         <f>$E$12</f>
@@ -24537,15 +24444,15 @@
       </c>
       <c r="E77" s="55" cm="1">
         <f t="array" ref="E77">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(E22,$E30,$E38,E45)</f>
-        <v>2002.762431581185</v>
+        <v>1001.3812157905925</v>
       </c>
       <c r="F77" s="55" cm="1">
         <f t="array" ref="F77">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(F22,$E30,$E38,F45)</f>
-        <v>70.727988893184005</v>
+        <v>35.363994446592002</v>
       </c>
       <c r="G77" s="55" cm="1">
         <f t="array" ref="G77">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(G22,$E30,$E38,G45)</f>
-        <v>102.15557769599998</v>
+        <v>51.07778884799999</v>
       </c>
       <c r="H77" s="2" t="str">
         <f>$E$12</f>
@@ -24557,15 +24464,15 @@
       </c>
       <c r="M77" s="55" cm="1">
         <f t="array" ref="M77">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(M22,$E30,$E38,E45)</f>
-        <v>2002.762431581185</v>
+        <v>1001.3812157905925</v>
       </c>
       <c r="N77" s="55" cm="1">
         <f t="array" ref="N77">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(N22,$E30,$E38,F45)</f>
-        <v>70.727988893184005</v>
+        <v>35.363994446592002</v>
       </c>
       <c r="O77" s="55" cm="1">
         <f t="array" ref="O77">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(O22,$E30,$E38,G45)</f>
-        <v>102.15557769599998</v>
+        <v>51.07778884799999</v>
       </c>
       <c r="P77" s="2" t="str">
         <f>$E$12</f>
@@ -24579,15 +24486,15 @@
       </c>
       <c r="E78" s="55" cm="1">
         <f t="array" ref="E78">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(E23,$E31,$E39,E46)</f>
-        <v>6344.3212597739548</v>
+        <v>3172.1606298869774</v>
       </c>
       <c r="F78" s="55" cm="1">
         <f t="array" ref="F78">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(F23,$E31,$E39,F46)</f>
-        <v>224.051078909952</v>
+        <v>112.025539454976</v>
       </c>
       <c r="G78" s="55" cm="1">
         <f t="array" ref="G78">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(G23,$E31,$E39,G46)</f>
-        <v>323.60693068799992</v>
+        <v>161.80346534399996</v>
       </c>
       <c r="H78" s="2" t="str">
         <f>$E$12</f>
@@ -24599,15 +24506,15 @@
       </c>
       <c r="M78" s="55" cm="1">
         <f t="array" ref="M78">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(M23,$E31,$E39,E46)</f>
-        <v>6344.3212597739548</v>
+        <v>3172.1606298869774</v>
       </c>
       <c r="N78" s="55" cm="1">
         <f t="array" ref="N78">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(N23,$E31,$E39,F46)</f>
-        <v>224.051078909952</v>
+        <v>112.025539454976</v>
       </c>
       <c r="O78" s="55" cm="1">
         <f t="array" ref="O78">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(O23,$E31,$E39,G46)</f>
-        <v>323.60693068799992</v>
+        <v>161.80346534399996</v>
       </c>
       <c r="P78" s="2" t="str">
         <f>$E$12</f>
@@ -24621,15 +24528,15 @@
       </c>
       <c r="E79" s="55" cm="1">
         <f t="array" ref="E79">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(E24,$E32,$E40,E47)</f>
-        <v>466.46466048000019</v>
+        <v>233.2323302400001</v>
       </c>
       <c r="F79" s="55" cm="1">
         <f t="array" ref="F79">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(F24,$E32,$E40,F47)</f>
-        <v>16.473300480000002</v>
+        <v>8.2366502400000012</v>
       </c>
       <c r="G79" s="55" cm="1">
         <f t="array" ref="G79">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(G24,$E32,$E40,G47)</f>
-        <v>23.793119999999995</v>
+        <v>11.896559999999997</v>
       </c>
       <c r="H79" s="2" t="str">
         <f>$E$12</f>
@@ -24641,15 +24548,15 @@
       </c>
       <c r="M79" s="55" cm="1">
         <f t="array" ref="M79">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(M24,$E32,$E40,E47)</f>
-        <v>466.46466048000019</v>
+        <v>233.2323302400001</v>
       </c>
       <c r="N79" s="55" cm="1">
         <f t="array" ref="N79">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(N24,$E32,$E40,F47)</f>
-        <v>16.473300480000002</v>
+        <v>8.2366502400000012</v>
       </c>
       <c r="O79" s="55" cm="1">
         <f t="array" ref="O79">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3(O24,$E32,$E40,G47)</f>
-        <v>23.793119999999995</v>
+        <v>11.896559999999997</v>
       </c>
       <c r="P79" s="2" t="str">
         <f>$E$12</f>
@@ -24663,7 +24570,7 @@
       </c>
       <c r="E81" s="111">
         <f>SUM(E77:G79)</f>
-        <v>9574.3563485022751</v>
+        <v>4787.1781742511375</v>
       </c>
       <c r="F81" s="112" t="str">
         <f>$E$12</f>
@@ -24674,7 +24581,7 @@
       </c>
       <c r="M81" s="111">
         <f>SUM(M77:O79)</f>
-        <v>9574.3563485022751</v>
+        <v>4787.1781742511375</v>
       </c>
       <c r="N81" s="112" t="str">
         <f>$E$12</f>
@@ -24691,7 +24598,7 @@
       <c r="G84" s="48"/>
       <c r="H84" s="48"/>
       <c r="I84" s="48"/>
-      <c r="J84" s="126"/>
+      <c r="J84" s="123"/>
       <c r="K84" s="48"/>
       <c r="L84" s="48"/>
       <c r="M84" s="48"/>
@@ -24701,9 +24608,9 @@
       <c r="Q84" s="48"/>
     </row>
     <row r="85" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D85" s="123" t="str">
-        <f>"Below are applications of " &amp; D61 &amp; " that are applied to the following contexts:"</f>
-        <v>Below are applications of VEERG 2026: 4.1.1.9, Equation (2) that are applied to the following contexts:</v>
+      <c r="D85" s="122" t="str">
+        <f>"Below are applications of " &amp; D6 &amp; " that are applied to the following contexts:"</f>
+        <v>Below are applications of VEERG 2026: 4.1.1.9, Equation (1) that are applied to the following contexts:</v>
       </c>
       <c r="E85" s="95"/>
       <c r="F85" s="95"/>
@@ -24711,619 +24618,326 @@
       <c r="H85" s="91"/>
     </row>
     <row r="86" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D86" s="124" t="s">
-        <v>279</v>
-      </c>
-      <c r="E86" s="122"/>
-      <c r="F86" s="122"/>
-      <c r="G86" s="122"/>
-      <c r="H86" s="125"/>
-    </row>
-    <row r="87" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D87" s="97" t="s">
-        <v>280</v>
-      </c>
-      <c r="E87" s="94"/>
-      <c r="F87" s="94"/>
-      <c r="G87" s="94"/>
-      <c r="H87" s="92"/>
-    </row>
-    <row r="88" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D86" s="97" t="s">
+        <v>270</v>
+      </c>
+      <c r="E86" s="94"/>
+      <c r="F86" s="94"/>
+      <c r="G86" s="94"/>
+      <c r="H86" s="92"/>
+    </row>
+    <row r="87" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D88" s="6" t="s">
+        <v>336</v>
+      </c>
+    </row>
     <row r="89" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D89" s="6" t="s">
-        <v>276</v>
+      <c r="D89" s="105" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="90" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D90" s="105" t="s">
-        <v>256</v>
+      <c r="D90" s="104" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="91" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D91" s="104" t="s">
-        <v>257</v>
+      <c r="D91" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="E91" s="54" t="s">
+        <v>148</v>
+      </c>
+      <c r="F91" s="54" t="s">
+        <v>149</v>
+      </c>
+      <c r="G91" s="54" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="92" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D92" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="E92" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="F92" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="G92" s="54" t="s">
-        <v>150</v>
+      <c r="D92" s="55" t="str">
+        <f>'Input - Feedlot'!$D$35</f>
+        <v>Solid storage</v>
+      </c>
+      <c r="E92" s="55">
+        <f>'Input - Feedlot'!E48</f>
+        <v>0.25</v>
+      </c>
+      <c r="F92" s="55">
+        <f>'Input - Feedlot'!F48</f>
+        <v>0.25</v>
+      </c>
+      <c r="G92" s="55">
+        <f>'Input - Feedlot'!G48</f>
+        <v>0.25</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="93" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D93" s="55" t="str">
+        <f>'Input - Feedlot'!$D$36</f>
+        <v>Composting (passive windrow)</v>
+      </c>
+      <c r="E93" s="55">
+        <f>'Input - Feedlot'!E53</f>
+        <v>0.25</v>
+      </c>
+      <c r="F93" s="55">
+        <f>'Input - Feedlot'!F53</f>
+        <v>0.25</v>
+      </c>
+      <c r="G93" s="55">
+        <f>'Input - Feedlot'!G53</f>
+        <v>0.25</v>
+      </c>
+      <c r="H93" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="94" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D94" s="55" t="str">
+        <f>'Input - Feedlot'!$D$41</f>
+        <v>Anaerobic lagoon</v>
+      </c>
+      <c r="E94" s="55">
+        <f>'Input - Feedlot'!E58</f>
+        <v>0.25</v>
+      </c>
+      <c r="F94" s="55">
+        <f>'Input - Feedlot'!F58</f>
+        <v>0.25</v>
+      </c>
+      <c r="G94" s="55">
+        <f>'Input - Feedlot'!G58</f>
+        <v>0.25</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="95" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D96" s="105" t="s">
+        <v>259</v>
+      </c>
+      <c r="L96" s="105" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="97" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D97" s="104" t="s">
+        <v>265</v>
+      </c>
+      <c r="L97" s="104" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="98" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D98" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="E98" s="54" t="s">
+        <v>148</v>
+      </c>
+      <c r="F98" s="54" t="s">
+        <v>149</v>
+      </c>
+      <c r="G98" s="54" t="s">
+        <v>150</v>
+      </c>
+      <c r="L98" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="M98" s="54" t="s">
+        <v>148</v>
+      </c>
+      <c r="N98" s="54" t="s">
+        <v>149</v>
+      </c>
+      <c r="O98" s="54" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="99" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D99" s="55" t="str">
         <f>'Input - Feedlot'!$D$35</f>
         <v>Solid storage</v>
       </c>
-      <c r="E93" s="55">
-        <f>'Input - Feedlot'!E48</f>
-        <v>0.25</v>
-      </c>
-      <c r="F93" s="55">
-        <f>'Input - Feedlot'!F48</f>
-        <v>0.25</v>
-      </c>
-      <c r="G93" s="55">
-        <f>'Input - Feedlot'!G48</f>
-        <v>0.25</v>
-      </c>
-      <c r="H93" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="94" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D94" s="55" t="str">
+      <c r="E99" s="55" cm="1">
+        <f t="array" ref="E99">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E22,$E$30,$E$38,E92)</f>
+        <v>1001.3812157905925</v>
+      </c>
+      <c r="F99" s="55" cm="1">
+        <f t="array" ref="F99">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F22,$E$30,$E$38,F92)</f>
+        <v>35.363994446592002</v>
+      </c>
+      <c r="G99" s="55" cm="1">
+        <f t="array" ref="G99">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G22,$E$30,$E$38,G92)</f>
+        <v>51.07778884799999</v>
+      </c>
+      <c r="H99" s="2" t="str">
+        <f>$E$12</f>
+        <v>kg N</v>
+      </c>
+      <c r="L99" s="55" t="str">
+        <f>'Input - Feedlot'!$D$35</f>
+        <v>Solid storage</v>
+      </c>
+      <c r="M99" s="55" cm="1">
+        <f t="array" ref="M99">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M22,$E$30,$E$38,E92)</f>
+        <v>1001.3812157905925</v>
+      </c>
+      <c r="N99" s="55" cm="1">
+        <f t="array" ref="N99">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N22,$E$30,$E$38,F92)</f>
+        <v>35.363994446592002</v>
+      </c>
+      <c r="O99" s="55" cm="1">
+        <f t="array" ref="O99">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O22,$E$30,$E$38,G92)</f>
+        <v>51.07778884799999</v>
+      </c>
+      <c r="P99" s="2" t="str">
+        <f>$E$12</f>
+        <v>kg N</v>
+      </c>
+    </row>
+    <row r="100" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D100" s="55" t="str">
         <f>'Input - Feedlot'!$D$36</f>
         <v>Composting (passive windrow)</v>
       </c>
-      <c r="E94" s="55">
-        <f>'Input - Feedlot'!E53</f>
-        <v>0.25</v>
-      </c>
-      <c r="F94" s="55">
-        <f>'Input - Feedlot'!F53</f>
-        <v>0.25</v>
-      </c>
-      <c r="G94" s="55">
-        <f>'Input - Feedlot'!G53</f>
-        <v>0.25</v>
-      </c>
-      <c r="H94" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="95" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D95" s="55" t="str">
-        <f>'Input - Feedlot'!$D$41</f>
-        <v>Anaerobic lagoon</v>
-      </c>
-      <c r="E95" s="55">
-        <f>'Input - Feedlot'!E58</f>
-        <v>0.25</v>
-      </c>
-      <c r="F95" s="55">
-        <f>'Input - Feedlot'!F58</f>
-        <v>0.25</v>
-      </c>
-      <c r="G95" s="55">
-        <f>'Input - Feedlot'!G58</f>
-        <v>0.25</v>
-      </c>
-      <c r="H95" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="96" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D97" s="105" t="s">
-        <v>259</v>
-      </c>
-      <c r="L97" s="105" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="98" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D98" s="104" t="s">
-        <v>265</v>
-      </c>
-      <c r="L98" s="104" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="99" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D99" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="E99" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="F99" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="G99" s="54" t="s">
-        <v>150</v>
-      </c>
-      <c r="L99" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="M99" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="N99" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="O99" s="54" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="100" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D100" s="55" t="str">
-        <f>'Input - Feedlot'!$D$35</f>
-        <v>Solid storage</v>
-      </c>
       <c r="E100" s="55" cm="1">
-        <f t="array" ref="E100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E22,$E$30,$E$38,E93)</f>
-        <v>1001.3812157905925</v>
+        <f t="array" ref="E100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E23,$E$31,$E$39,E93)</f>
+        <v>3172.1606298869774</v>
       </c>
       <c r="F100" s="55" cm="1">
-        <f t="array" ref="F100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F22,$E$30,$E$38,F93)</f>
-        <v>35.363994446592002</v>
+        <f t="array" ref="F100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F23,$E$31,$E$39,F93)</f>
+        <v>112.025539454976</v>
       </c>
       <c r="G100" s="55" cm="1">
-        <f t="array" ref="G100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G22,$E$30,$E$38,G93)</f>
-        <v>51.07778884799999</v>
+        <f t="array" ref="G100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G23,$E$31,$E$39,G93)</f>
+        <v>161.80346534399996</v>
       </c>
       <c r="H100" s="2" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
       <c r="L100" s="55" t="str">
-        <f>'Input - Feedlot'!$D$35</f>
-        <v>Solid storage</v>
+        <f>'Input - Feedlot'!$D$36</f>
+        <v>Composting (passive windrow)</v>
       </c>
       <c r="M100" s="55" cm="1">
-        <f t="array" ref="M100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M22,$E$30,$E$38,E93)</f>
-        <v>1001.3812157905925</v>
+        <f t="array" ref="M100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M23,$E$31,$E$39,E93)</f>
+        <v>3172.1606298869774</v>
       </c>
       <c r="N100" s="55" cm="1">
-        <f t="array" ref="N100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N22,$E$30,$E$38,F93)</f>
-        <v>35.363994446592002</v>
+        <f t="array" ref="N100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N23,$E$31,$E$39,F93)</f>
+        <v>112.025539454976</v>
       </c>
       <c r="O100" s="55" cm="1">
-        <f t="array" ref="O100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O22,$E$30,$E$38,G93)</f>
-        <v>51.07778884799999</v>
+        <f t="array" ref="O100">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O23,$E$31,$E$39,G93)</f>
+        <v>161.80346534399996</v>
       </c>
       <c r="P100" s="2" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
     </row>
-    <row r="101" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D101" s="55" t="str">
-        <f>'Input - Feedlot'!$D$36</f>
-        <v>Composting (passive windrow)</v>
+        <f>'Input - Feedlot'!$D$41</f>
+        <v>Anaerobic lagoon</v>
       </c>
       <c r="E101" s="55" cm="1">
-        <f t="array" ref="E101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E23,$E$31,$E$39,E94)</f>
-        <v>3172.1606298869774</v>
+        <f t="array" ref="E101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E24,$E$32,$E$40,E94)</f>
+        <v>233.2323302400001</v>
       </c>
       <c r="F101" s="55" cm="1">
-        <f t="array" ref="F101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F23,$E$31,$E$39,F94)</f>
-        <v>112.025539454976</v>
+        <f t="array" ref="F101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F24,$E$32,$E$40,F94)</f>
+        <v>8.2366502400000012</v>
       </c>
       <c r="G101" s="55" cm="1">
-        <f t="array" ref="G101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G23,$E$31,$E$39,G94)</f>
-        <v>161.80346534399996</v>
+        <f t="array" ref="G101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G24,$E$32,$E$40,G94)</f>
+        <v>11.896559999999997</v>
       </c>
       <c r="H101" s="2" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
       <c r="L101" s="55" t="str">
-        <f>'Input - Feedlot'!$D$36</f>
-        <v>Composting (passive windrow)</v>
+        <f>'Input - Feedlot'!$D$41</f>
+        <v>Anaerobic lagoon</v>
       </c>
       <c r="M101" s="55" cm="1">
-        <f t="array" ref="M101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M23,$E$31,$E$39,E94)</f>
-        <v>3172.1606298869774</v>
+        <f t="array" ref="M101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M24,$E$32,$E$40,E94)</f>
+        <v>233.2323302400001</v>
       </c>
       <c r="N101" s="55" cm="1">
-        <f t="array" ref="N101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N23,$E$31,$E$39,F94)</f>
-        <v>112.025539454976</v>
+        <f t="array" ref="N101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N24,$E$32,$E$40,F94)</f>
+        <v>8.2366502400000012</v>
       </c>
       <c r="O101" s="55" cm="1">
-        <f t="array" ref="O101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O23,$E$31,$E$39,G94)</f>
-        <v>161.80346534399996</v>
+        <f t="array" ref="O101">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O24,$E$32,$E$40,G94)</f>
+        <v>11.896559999999997</v>
       </c>
       <c r="P101" s="2" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
     </row>
-    <row r="102" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D102" s="55" t="str">
-        <f>'Input - Feedlot'!$D$41</f>
-        <v>Anaerobic lagoon</v>
-      </c>
-      <c r="E102" s="55" cm="1">
-        <f t="array" ref="E102">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E24,$E$32,$E$40,E95)</f>
-        <v>233.2323302400001</v>
-      </c>
-      <c r="F102" s="55" cm="1">
-        <f t="array" ref="F102">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F24,$E$32,$E$40,F95)</f>
-        <v>8.2366502400000012</v>
-      </c>
-      <c r="G102" s="55" cm="1">
-        <f t="array" ref="G102">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G24,$E$32,$E$40,G95)</f>
-        <v>11.896559999999997</v>
-      </c>
-      <c r="H102" s="2" t="str">
+    <row r="102" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D103" s="110" t="s">
+        <v>271</v>
+      </c>
+      <c r="E103" s="111">
+        <f>SUM(E99:G101)</f>
+        <v>4787.1781742511375</v>
+      </c>
+      <c r="F103" s="112" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
-      <c r="L102" s="55" t="str">
-        <f>'Input - Feedlot'!$D$41</f>
-        <v>Anaerobic lagoon</v>
-      </c>
-      <c r="M102" s="55" cm="1">
-        <f t="array" ref="M102">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M24,$E$32,$E$40,E95)</f>
-        <v>233.2323302400001</v>
-      </c>
-      <c r="N102" s="55" cm="1">
-        <f t="array" ref="N102">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N24,$E$32,$E$40,F95)</f>
-        <v>8.2366502400000012</v>
-      </c>
-      <c r="O102" s="55" cm="1">
-        <f t="array" ref="O102">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O24,$E$32,$E$40,G95)</f>
-        <v>11.896559999999997</v>
-      </c>
-      <c r="P102" s="2" t="str">
+      <c r="L103" s="110" t="s">
+        <v>271</v>
+      </c>
+      <c r="M103" s="111">
+        <f>SUM(M99:O101)</f>
+        <v>4787.1781742511375</v>
+      </c>
+      <c r="N103" s="112" t="str">
         <f>$E$12</f>
         <v>kg N</v>
       </c>
     </row>
-    <row r="103" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D104" s="110" t="s">
-        <v>281</v>
-      </c>
-      <c r="E104" s="111">
-        <f>SUM(E100:G102)</f>
-        <v>4787.1781742511375</v>
-      </c>
-      <c r="F104" s="112" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-      <c r="L104" s="110" t="s">
-        <v>281</v>
-      </c>
-      <c r="M104" s="111">
-        <f>SUM(M100:O102)</f>
-        <v>4787.1781742511375</v>
-      </c>
-      <c r="N104" s="112" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-    </row>
-    <row r="105" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C107" s="48"/>
-      <c r="D107" s="48"/>
-      <c r="E107" s="48"/>
-      <c r="F107" s="48"/>
-      <c r="G107" s="48"/>
-      <c r="H107" s="48"/>
-      <c r="I107" s="48"/>
-      <c r="K107" s="48"/>
-      <c r="L107" s="48"/>
-      <c r="M107" s="48"/>
-      <c r="N107" s="48"/>
-      <c r="O107" s="48"/>
-      <c r="P107" s="48"/>
-      <c r="Q107" s="48"/>
-    </row>
-    <row r="108" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D108" s="6" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="109" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D109" s="105" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="110" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D110" s="104" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="111" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D111" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="E111" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="F111" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="G111" s="54" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="112" spans="3:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D112" s="55" t="str">
-        <f>'Input - Feedlot'!$D$35</f>
-        <v>Solid storage</v>
-      </c>
-      <c r="E112" s="55">
-        <f>'Input - Feedlot'!E47</f>
-        <v>0.25</v>
-      </c>
-      <c r="F112" s="55">
-        <f>'Input - Feedlot'!F47</f>
-        <v>0.25</v>
-      </c>
-      <c r="G112" s="55">
-        <f>'Input - Feedlot'!G47</f>
-        <v>0.25</v>
-      </c>
-      <c r="H112" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="113" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D113" s="55" t="str">
-        <f>'Input - Feedlot'!$D$36</f>
-        <v>Composting (passive windrow)</v>
-      </c>
-      <c r="E113" s="55">
-        <f>'Input - Feedlot'!E52</f>
-        <v>0.25</v>
-      </c>
-      <c r="F113" s="55">
-        <f>'Input - Feedlot'!F52</f>
-        <v>0.25</v>
-      </c>
-      <c r="G113" s="55">
-        <f>'Input - Feedlot'!G52</f>
-        <v>0.25</v>
-      </c>
-      <c r="H113" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="114" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D114" s="55" t="str">
-        <f>'Input - Feedlot'!$D$41</f>
-        <v>Anaerobic lagoon</v>
-      </c>
-      <c r="E114" s="55">
-        <f>'Input - Feedlot'!E57</f>
-        <v>0.25</v>
-      </c>
-      <c r="F114" s="55">
-        <f>'Input - Feedlot'!F57</f>
-        <v>0.25</v>
-      </c>
-      <c r="G114" s="55">
-        <f>'Input - Feedlot'!G57</f>
-        <v>0.25</v>
-      </c>
-      <c r="H114" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="115" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D116" s="105" t="s">
-        <v>272</v>
-      </c>
-      <c r="L116" s="105" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="117" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D117" s="104" t="s">
-        <v>275</v>
-      </c>
-      <c r="L117" s="104" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="118" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D118" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="E118" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="F118" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="G118" s="54" t="s">
-        <v>150</v>
-      </c>
-      <c r="L118" s="54" t="s">
-        <v>68</v>
-      </c>
-      <c r="M118" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="N118" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="O118" s="54" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="119" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D119" s="55" t="str">
-        <f>'Input - Feedlot'!$D$35</f>
-        <v>Solid storage</v>
-      </c>
-      <c r="E119" s="55" cm="1">
-        <f t="array" ref="E119">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E22,$E$30,$E$38,E112)</f>
-        <v>1001.3812157905925</v>
-      </c>
-      <c r="F119" s="55" cm="1">
-        <f t="array" ref="F119">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F22,$E$30,$E$38,F112)</f>
-        <v>35.363994446592002</v>
-      </c>
-      <c r="G119" s="55" cm="1">
-        <f t="array" ref="G119">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G22,$E$30,$E$38,G112)</f>
-        <v>51.07778884799999</v>
-      </c>
-      <c r="H119" s="2" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-      <c r="L119" s="55" t="str">
-        <f>'Input - Feedlot'!$D$35</f>
-        <v>Solid storage</v>
-      </c>
-      <c r="M119" s="55" cm="1">
-        <f t="array" ref="M119">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M22,$E$30,$E$38,E112)</f>
-        <v>1001.3812157905925</v>
-      </c>
-      <c r="N119" s="55" cm="1">
-        <f t="array" ref="N119">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N22,$E$30,$E$38,F112)</f>
-        <v>35.363994446592002</v>
-      </c>
-      <c r="O119" s="55" cm="1">
-        <f t="array" ref="O119">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O22,$E$30,$E$38,G112)</f>
-        <v>51.07778884799999</v>
-      </c>
-      <c r="P119" s="2" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-    </row>
-    <row r="120" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D120" s="55" t="str">
-        <f>'Input - Feedlot'!$D$36</f>
-        <v>Composting (passive windrow)</v>
-      </c>
-      <c r="E120" s="55" cm="1">
-        <f t="array" ref="E120">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E23,$E$31,$E$39,E113)</f>
-        <v>3172.1606298869774</v>
-      </c>
-      <c r="F120" s="55" cm="1">
-        <f t="array" ref="F120">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F23,$E$31,$E$39,F113)</f>
-        <v>112.025539454976</v>
-      </c>
-      <c r="G120" s="55" cm="1">
-        <f t="array" ref="G120">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G23,$E$31,$E$39,G113)</f>
-        <v>161.80346534399996</v>
-      </c>
-      <c r="H120" s="2" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-      <c r="L120" s="55" t="str">
-        <f>'Input - Feedlot'!$D$36</f>
-        <v>Composting (passive windrow)</v>
-      </c>
-      <c r="M120" s="55" cm="1">
-        <f t="array" ref="M120">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M23,$E$31,$E$39,E113)</f>
-        <v>3172.1606298869774</v>
-      </c>
-      <c r="N120" s="55" cm="1">
-        <f t="array" ref="N120">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N23,$E$31,$E$39,F113)</f>
-        <v>112.025539454976</v>
-      </c>
-      <c r="O120" s="55" cm="1">
-        <f t="array" ref="O120">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O23,$E$31,$E$39,G113)</f>
-        <v>161.80346534399996</v>
-      </c>
-      <c r="P120" s="2" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-    </row>
-    <row r="121" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D121" s="55" t="str">
-        <f>'Input - Feedlot'!$D$41</f>
-        <v>Anaerobic lagoon</v>
-      </c>
-      <c r="E121" s="55" cm="1">
-        <f t="array" ref="E121">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(E24,$E$32,$E$40,E114)</f>
-        <v>233.2323302400001</v>
-      </c>
-      <c r="F121" s="55" cm="1">
-        <f t="array" ref="F121">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(F24,$E$32,$E$40,F114)</f>
-        <v>8.2366502400000012</v>
-      </c>
-      <c r="G121" s="55" cm="1">
-        <f t="array" ref="G121">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(G24,$E$32,$E$40,G114)</f>
-        <v>11.896559999999997</v>
-      </c>
-      <c r="H121" s="2" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-      <c r="L121" s="55" t="str">
-        <f>'Input - Feedlot'!$D$41</f>
-        <v>Anaerobic lagoon</v>
-      </c>
-      <c r="M121" s="55" cm="1">
-        <f t="array" ref="M121">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(M24,$E$32,$E$40,E114)</f>
-        <v>233.2323302400001</v>
-      </c>
-      <c r="N121" s="55" cm="1">
-        <f t="array" ref="N121">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(N24,$E$32,$E$40,F114)</f>
-        <v>8.2366502400000012</v>
-      </c>
-      <c r="O121" s="55" cm="1">
-        <f t="array" ref="O121">MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1(O24,$E$32,$E$40,G114)</f>
-        <v>11.896559999999997</v>
-      </c>
-      <c r="P121" s="2" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-    </row>
-    <row r="122" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D123" s="110" t="s">
-        <v>278</v>
-      </c>
-      <c r="E123" s="111">
-        <f>SUM(E119:G121)</f>
-        <v>4787.1781742511375</v>
-      </c>
-      <c r="F123" s="112" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-      <c r="L123" s="110" t="s">
-        <v>278</v>
-      </c>
-      <c r="M123" s="111">
-        <f>SUM(M119:O121)</f>
-        <v>4787.1781742511375</v>
-      </c>
-      <c r="N123" s="112" t="str">
-        <f>$E$12</f>
-        <v>kg N</v>
-      </c>
-    </row>
-    <row r="124" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="4:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="113" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="114" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="115" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="116" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="117" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="118" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="119" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="120" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="121" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="122" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="123" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="124" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="125" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="126" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="127" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="128" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="129" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="130" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="131" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -25620,10 +25234,10 @@
         <v>118</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="M25" s="1"/>
     </row>
@@ -25638,10 +25252,10 @@
         <v>82</v>
       </c>
       <c r="G27" s="39" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="J27" s="39" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="M27" s="1"/>
     </row>
@@ -25659,7 +25273,7 @@
         <v>Crop</v>
       </c>
       <c r="J28" s="39" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="M28" s="1"/>
     </row>
@@ -25677,7 +25291,7 @@
         <v>Pasture</v>
       </c>
       <c r="J29" s="39" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="M29" s="1"/>
     </row>
@@ -25691,7 +25305,7 @@
         <v>Composting (passive windrow) (m=6)</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="M30" s="1"/>
     </row>
@@ -25705,7 +25319,7 @@
         <v>Direct application (m=13)</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="M31" s="1"/>
     </row>
@@ -25719,7 +25333,7 @@
         <v>Anaerobic lagoon (m=1)</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="M32" s="1"/>
     </row>
@@ -26669,7 +26283,7 @@
         <f t="array" ref="H89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.03</v>
       </c>
-      <c r="I89" s="138" t="str" cm="1">
+      <c r="I89" s="135" t="str" cm="1">
         <f t="array" ref="I89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26685,7 +26299,7 @@
         <f t="array" ref="L89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.01</v>
       </c>
-      <c r="M89" s="138" t="str" cm="1">
+      <c r="M89" s="135" t="str" cm="1">
         <f t="array" ref="M89">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26715,7 +26329,7 @@
         <f t="array" ref="H90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.02</v>
       </c>
-      <c r="I90" s="138" t="str" cm="1">
+      <c r="I90" s="135" t="str" cm="1">
         <f t="array" ref="I90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26731,7 +26345,7 @@
         <f t="array" ref="L90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.02</v>
       </c>
-      <c r="M90" s="138" t="str" cm="1">
+      <c r="M90" s="135" t="str" cm="1">
         <f t="array" ref="M90">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26761,7 +26375,7 @@
         <f t="array" ref="H91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.01</v>
       </c>
-      <c r="I91" s="138" t="str" cm="1">
+      <c r="I91" s="135" t="str" cm="1">
         <f t="array" ref="I91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26777,7 +26391,7 @@
         <f t="array" ref="L91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.01</v>
       </c>
-      <c r="M91" s="138" t="str" cm="1">
+      <c r="M91" s="135" t="str" cm="1">
         <f t="array" ref="M91">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26807,7 +26421,7 @@
         <f t="array" ref="H92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0</v>
       </c>
-      <c r="I92" s="138" t="str" cm="1">
+      <c r="I92" s="135" t="str" cm="1">
         <f t="array" ref="I92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26823,7 +26437,7 @@
         <f t="array" ref="L92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0</v>
       </c>
-      <c r="M92" s="138" t="str" cm="1">
+      <c r="M92" s="135" t="str" cm="1">
         <f t="array" ref="M92">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26853,7 +26467,7 @@
         <f t="array" ref="H93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.77</v>
       </c>
-      <c r="I93" s="138" t="str" cm="1">
+      <c r="I93" s="135" t="str" cm="1">
         <f t="array" ref="I93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26869,7 +26483,7 @@
         <f t="array" ref="L93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>0.77</v>
       </c>
-      <c r="M93" s="138" t="str" cm="1">
+      <c r="M93" s="135" t="str" cm="1">
         <f t="array" ref="M93">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</f>
         <v>No data</v>
       </c>
@@ -26880,10 +26494,10 @@
     </row>
     <row r="94" spans="4:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I94" s="1" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="M94" s="24" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
     </row>
     <row r="95" spans="4:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -27705,6 +27319,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -27899,16 +27522,11 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAIgAsACIAdABlAHgAdAAiADoAIgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGwAbwBzAHQAIABpAG4AIAB0AGgAZQAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkAGwAbwB0ACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAFMATABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA1ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AG8AIABlAGEAYwBoACAAdABlAHIAdABpAGEAcgB5ACAAcwB5AHMAdABlAG0AIABhAHMAcwB1AG0AZQBkACAAdABoAGEAdAAgADIAIABwAGUAcgAgAGMAZQBuAHQAIABpAHMAIAByAHUAbgAgAC0AIABvAGYAZgAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAZQBlAGQAIABwAGEAZAAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AG8AIABlAGEAYwBoACAAdABlAHIAdABpAGEAcgB5ACAAcwB5AHMAdABlAG0AIABhAHMAcwB1AG0AZQBkACAAdABoAGEAdAAgADIAIABwAGUAcgAgAGMAZQBuAHQAIABpAHMAIAByAHUAbgAgAC0AIABvAGYAZgAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAZQBlAGQAIABwAGEAZAAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAG0AMQBUADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AFwAbgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA2ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4ATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBtADMAIABDAEgANAAgAC8AIABrAGcAIABWAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA5ACkAOwBcAG4AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAxAE0ATQBTAE8AcAB0AGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAE0ATQBTAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBTAHQAYQBnAGUAMwBNAE0AUwBPAHAAdABpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBMAGkAdgBlAHMAdABvAGMAawBDAGwAYQBzAHMAZQBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQB4AHAAbwByAHQAIABtAGkAZAAgAGYAZQBkAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAeABwAG8AcgB0ACAAbABvAG4AZwAgAGYAZQBkAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgAxADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIAAoAGQAYQB5AHMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAKABkAGEAeQBzACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADEAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgACgAZABhAHkAcwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIATABlAG4AZwB0AGgAIABvAGYAIABTAHQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIAMQAtADgAMAAgAGQAYQB5AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIAOAAxAC0AMgAwADAAIABkAGEAeQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIAMgAwADEAKwAgAGQAYQB5AHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADIAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEEAbgBpAG0AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgAyADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEEAbgBpAG0AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAHYAZQBkACAAZgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAcwAgAHQAbwAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBhAG0AZQBkACAAXAB1ADAAMAAyADcAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAAtACAAbwByAGkAZwBpAG4AYQBsACAAaABhAHMAIABoAGUAYQBkAGUAcgAgAFwAdQAwADAAMgA3AFUAbgBpAHQAXAB1ADAAMAAyADcAIAB3AGgAaQBjAGgAIABjAG8AdgBlAHIAcwAgAHQAdwBvACAAYwBvAGwAdQBtAG4AcwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADAALAAgADcALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBlAGQAbABvAHQAIAB0AHkAcABlAFwAIgAsACAAXAAiAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBcACIALAAgAFwAIgBVAG4AaQB0AFwAIgAsACAAXAAiADIAMAAwADUALQAyADAAMAA5AFwAIgAsACAAXAAiADIAMAAxADAALQAyADAAMQA0AFwAIgAsACAAXAAiADIAMAAxADUALQAyADAAMQA5AFwAIgAsACAAXAAiADIAMAAyADAALQAyADAAMgAzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARABhAHkAcwAgAG8AbgAgAGYAZQBlAGQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgADcAMAAsACAANwAwACwAIAA3ADAALAAgADcANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAMQAwAC4AMAAsACAAMQAwAC4AMAAsACAAMQAwAC4ANAAsACAAMQAwAC4ANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIATgAgAHIAZQB0AGUAbgB0AGkAbwBuAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdAAgAG8AZgAgAGkAbgB0AGEAawBlAFwAIgAsACAAMgAxAC4AMQAsACAAMgAwAC4ANAAsACAAMgAwAC4ANAAsACAAMgAwAC4ANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEQAYQB5AHMAIABvAG4AIABmAGUAZQBkAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIAAxADEANQAsACAAMQAxADUALAAgADEAMgAwACwAIAAxADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBkAGEAeQBcACIALAAgADEAMQAuADIALAAgADEAMAAuADgALAAgADEAMAAuADgALAAgADEAMAAuADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBOACAAcgBlAHQAZQBuAHQAaQBvAG4AXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0ACAAbwBmACAAaQBuAHQAYQBrAGUAXAAiACwAIAAxADIALgA1ACwAIAAxADIALgA3ACwAIAAxADIALgA3ACwAIAAxADIALgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgBEAGEAeQBzACAAbwBuACAAZgBlAGUAZABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAMgA1ADAALAAgADIANQAwACwAIAAyADUAMAAsACAAMgA1ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBkAGEAeQBcACIALAAgADkALgAwACwAIAA4AC4ANQAsACAAOAAuADIALAAgADgALgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgBOACAAcgBlAHQAZQBuAHQAaQBvAG4AXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0ACAAbwBmACAAaQBuAHQAYQBrAGUAXAAiACwAIAA2AC4ANgAsACAANwAuADAALAAgADcALgAwACwAIAA3AC4AMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADMAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARABpAGUAdAAgAHAAcgBvAHAAZQByAHQAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARABpAGUAdAAgAHAAcgBvAHAAZQByAHQAaQBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADMAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARABpAGUAdAAgAHAAcgBvAHAAZQByAHQAaQBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AEMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAZgByAGEAYwB0AGkAbwBuACAAYwBvAGwAdQBtAG4AIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAATgBEAEYAIABhAG4AZAAgAEUAdABoAGUAcgAgAGUAeAB0AHIAYQBjAHQAIAB2AGEAbAB1AGUAcwAgAHQAbwAgAGYAcgBhAGMAdABpAG8AbgBzAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwB2AGUAZAAgAGYAZQBlAGQAbABvAHQAIAB0AHkAcABlAHMAIAB0AG8AIABhACAAcwBlAHAAYQByAGEAdABlACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADgALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBlAGQAbABvAHQAIAB0AHkAcABlAFwAIgAsACAAXAAiAE4AdQB0AHIAaQBlAG4AdAAgAGEAbgBhAGwAeQBzAGkAcwBcACIALAAgAFwAIgBVAG4AaQB0AFwAIgAsACAAXAAiADIAMAAwADUALQAyADAAMAA5AFwAIgAsACAAXAAiADIAMAAxADAALQAyADAAMQA0AFwAIgAsACAAXAAiADIAMAAxADUALQAyADAAMQA5AFwAIgAsACAAXAAiADIAMAAyADAALQAyADAAMgAzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAZgByAGEAYwB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBOAEQARgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAAyADMALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAwAC4AMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBFAHQAaABlAHIAIABFAHgAdAByAGEAYwB0AFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADQALgA1ACwAIAA0AC4ANQAsACAANAAuADgALAAgADQALgA4ACwAIAAwAC4AMAA0ADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQAzACwAIAAwAC4AMQAyADUALAAgADAALgAxADIALAAgADAALgAxADIALAAgADAALgAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBOAEQARgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAAyADQALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAwAC4AMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARQB0AGgAZQByACAARQB4AHQAcgBhAGMAdABcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAA1AC4AMAAsACAANQAuADAALAAgADUALgAwACwAIAA1AC4AMAAsACAAMAAuADAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQAzACwAIAAwAC4AMQAyADUALAAgADAALgAxADIALAAgADAALgAxADIALAAgADAALgAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAE4ARABGAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADIANAAuADAALAAgADIANAAuADAALAAgADIANAAuADAALAAgADIANAAuADAALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAEUAdABoAGUAcgAgAEUAeAB0AHIAYQBjAHQAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAANQAuADAALAAgADUALgAwACwAIAA1AC4ANQAsACAANQAuADUALAAgADAALgAwADUANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADQAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQBUACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABNAEMARgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANAA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHUAcABsAGkAYwBhAHQAZQBkACAATgBTAFcAIAB2AGEAbAB1AGUAcwAgAGYAbwByACAAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAE4AVAAgAGEAbgBkACAAVABBAFMAIABjAG8AbAB1AG0AbgBzACAAdwBpAHQAaAAgAFwAdQAwADAAMgA3AG4AbwAgAGQAYQB0AGEAXAB1ADAAMAAyADcAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMQAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAE4AUwBXAFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAE4AVABcACIALAAgAFwAIgBTAEEAXAAiACwAIABcACIAVgBJAEMAXAAiACwAIABcACIAVwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAzACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBOAG8AIABkAGEAdABhAFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlACAAKABTAHQAbwBjAGsAcABpAGwAZQApAFwAIgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAXAAiAE4AbwAgAGQAYQB0AGEAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBOAG8AIABkAGEAdABhAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAMAAsACAAMAAsACAAXAAiAE4AbwAgAGQAYQB0AGEAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAcgB0AGkAYQByAHkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAKABFAGYAZgBsAHUAZQBuAHQAIABwAG8AbgBkACkAXAAiACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA3ACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgAFwAIgBOAG8AIABkAGEAdABhAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADUAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzACAAKABFAEYAbQBUACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgA1ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgACgARQBGAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAE0ATQBTACAAbgBhAG0AZQBzACAAdABoAGEAdAAgAG0AYQB0AGMAaAAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAVABcACIALAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AVAAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4AMAAwADUANAAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQAgACgAUwB0AG8AYwBrAHAAaQBsAGUAKQBcACIALAAgADAALgAwADAANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4AMAAxACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAcgB0AGkAYQByAHkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAKABFAGYAZgBsAHUAZQBuAHQAIABQAG8AbgBkACkAXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgA2ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwAgACgARgByAGEAYwBHAEEAUwBNAG0AVAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgA2ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwAgACgARgByAGEAYwBHAEEAUwBNAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEYAcgBhAGMARwBBAFMATQBtAFQAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAaQBtAGEAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAbABvAHQAIAAoAEYAZQBlAGQAcABhAGQAKQBcACIALAAgADAALgA2ACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlACAAKABTAHQAbwBjAGsAcABpAGwAZQApAFwAIgAsACAAMAAuADIANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4ANAAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAHIAdABpAGEAcgB5AFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAApAFwAIgAsACAAMAAuADMANQAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEAOgAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4AMQAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAE0AYQBuAHUAcgBlACAATQBlAHQAaABhAG4AZQAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAXwBDAEgANABcAG4AdAAgAEMASAA0AFwAbgB7AEUAfQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgARABfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABOAF8AewBqAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXABuAEQAXwBqACAAPQAgAGwAZQBuAGcAdABoACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIABkAGEAeQBzAFwAbgBNAF8AagBtAFQAIAA9ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABwAGUAcgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACwAIABNAE0AUwAsACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADoAIABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAaABlAGEAZABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABfAGoALAAgAE0AXwBqAG0AVAAsACAATgBfAGoALABcAG4AIAAgACAAIAAoAEQAXwBqACAAKgAgAE0AXwBqAG0AVAAgACoAIABOAF8AagApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAEgANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHsARQB9AF8AewBDAEgANAB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABEAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAE4AXwB7AGoAfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqAFwAIgAsAFwAIgBsAGUAbgBnAHQAaAAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAZABhAHkAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAbQBUAFwAIgAsAFwAIgBtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAHAAZQByACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAALAAgAE0ATQBTACwAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAOgAgAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALABcACIAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAaABlAGEAZABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AFwAbgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAE0ATQBTAFwAbgBNAF8AagBtADUAVAAxAFwAbgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBfAHsAagBtAD0ANQAsAFQAPQAxAH0APQBWAFMAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAAQgBPAFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAD0ANQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXABuAFYAUwBfAGoAIAA9ACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4AQgBPACAAPQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAIAA6ACAAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXABuAE0ATQBTAF8AbQA1AFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBNAEMARgBfAGkAbQA1ACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGQAcgB5AGwAbwB0ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAFMAXwBqACwAIABCAE8ALAAgAE0ATQBTAF8AbQA1AFQAMQAsACAATQBDAEYAXwBpAG0ANQAsACAAcgBoAG8ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIABNAEMARgBfAGkAbQA1ACwAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABNAEMARgBfAGkAbQA1ACkALAAgAE0AQwBGAF8AaQBtADUALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIABWAFMAXwBqACAAKgAgAEIATwAgACoAIABNAE0AUwBfAG0ANQBUADEAIAAqACAATQBDAEYAXwBpAG0ANQAgACoAIAByAGgAbwBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAbQA1AFQAMQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAagBtAD0ANQAsAFQAPQAxAH0APQBWAFMAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAAQgBPAFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAD0ANQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAG0ANQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtADUAXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGQAcgB5AGwAbwB0ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAGgAbwBcACIALABcACIAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAA6ACAAawBnAC8AbQAzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAFwAIgAsACAAXAAiAHMAdABhAHQAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAbgBNAF8AagBtAFQAMgBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGoAbQBUAD0AMgB9AD0AKAAxAC0AVgBTAEwAKQBcAFwAdABpAG0AZQBzACAAVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXABuAFYAUwBMACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AVgBTAF8AagAgAD0AIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBCAE8AIAA9ACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgADoAIABtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcAG4ATQBNAFMAXwBtAFQAMgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ATQBDAEYAXwBpAG0AIAA9ACAAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgAGEAbgBkACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAFMATAAsACAAVgBTAF8AagAsACAAQgBPACwAIABNAE0AUwBfAG0AVAAyACwAIABNAEMARgBfAGkAbQAsACAAcgBoAG8ALABcAG4AIAAgACAAIAAoADEAIAAtACAAVgBTAEwAKQAgACoAIABWAFMAXwBqACAAKgAgAEIATwAgACoAIABNAE0AUwBfAG0AVAAyACAAKgAgAE0AQwBGAF8AaQBtACAAKgAgAHIAaABvAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGoAbQBUAD0AMgB9AD0AKAAxAC0AVgBTAEwAKQBcAFwAdABpAG0AZQBzACAAVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAEwAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAG0AVAAyAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBDAEYAXwBpAG0AXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAE0ATQBTACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAOgAgAGsAZwAvAG0AMwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAaQBcACIALAAgAFwAIgBzAHQAYQB0AGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBcAG4AUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADMAIABNAE0AUwBcAG4ATQBfAGoAbQAxAFQAMwBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGoAbQA9ADEALABUAD0AMwB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0APQAxACwAVAA9ADMAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQA9ADEAfQBcAFwAdABpAG0AZQBzACAAXABcAHIAaABvAFwAbgBWAFMAXwBqACAAPQAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAEIATwAgAD0AIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAbgBNAE0AUwBfAG0AMQBUADMAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIAB0AG8AIAB0AGUAcgB0AGkAYQByAHkAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBNAEMARgBfAGkAbQAxACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAHIAaABvACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAOgAgAGsAZwAvAG0AMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAUwBfAGoALAAgAEIATwAsACAATQBNAFMAXwBtADEAVAAzACwAIABNAEMARgBfAGkAbQAxACwAIAByAGgAbwAsAFwAbgAgACAAIAAgAFYAUwBfAGoAIAAqACAAQgBPACAAKgAgAE0ATQBTAF8AbQAxAFQAMwAgACoAIABNAEMARgBfAGkAbQAxACAAKgAgAHIAaABvAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADMAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAbQAxAFQAMwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANAApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAagBtAD0AMQAsAFQAPQAzAH0APQBWAFMAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAAQgBPAFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAbQA9ADEALABUAD0AMwB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAagAgADoAIABrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIATwBcACIALABcACIAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgADoAIABtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBtADEAVAAzAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAHQAbwAgAHQAZQByAHQAaQBhAHIAeQAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtADEAXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsAFwAIgBkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAFYAUwBfAGoAXABuAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4AVgBTAF8AewBqAH0APQBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAoADEALQBEAE0ARABfAHsAagB9ACkAXABcAHQAaQBtAGUAcwAoADEALQBBACkAXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABpAG4AdABhAGsAZQAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAEQATQBEAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAEEAIAA9ACAAYQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALAAgAEQATQBEAF8AagAsACAAQQAsAFwAbgAgACAAIAAgAEkAXwBqACAAKgAgACgAMQAgAC0AIABEAE0ARABfAGoAKQAgACoAIAAoADEAIAAtACAAQQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBTAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBfAHsAagB9AD0ASQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARABNAEQAXwB7AGoAfQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AQQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAXwBqAFwAIgAsAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIABqACAAOgAgAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgAGoAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAFwAIgAsAFwAIgBhAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgAxADoAIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEALgAxAC4AOQAgAE0AYQBuAHUAcgBlACAAQQBwAHAAbABpAGUAZAAgAHQAbwAgAFMAbwBpAGwAcwBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAxAFwAbgBrAGcAIABOAFwAbgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADEAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAA9ADIALAAzAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIALAAzAH0ALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0AVAA9ADIALAAzAH0AKQApAFwAXAB0AGkAbQBlAHMAIABQAEYAXABuAE0ATgBfAGoAbQBUADIAMwAgAD0AIABtAGEAcwBzACAAbwBmACAATgAgAGkAbgAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAYQBuAGQAIAB0AGUAcgB0AGkAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAcwB0AGEAZwBlAHMAIABhAHMAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIAA6ACAAawBnACAATgBcAG4ARQBGAF8AbQBUADIAMwAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAbgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGEAbgBpAG0AYQBsACAAdwBhAHMAdABlACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgAGYAbwByACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcAG4AUABGACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAZgBlAGUAZABsAG8AdAAgAGIAbwB1AG4AZABhAHIAeQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtAFQAMgAzACwAIABFAEYAXwBtAFQAMgAzACwAIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzACwAIABQAEYALABcAG4AIAAgACAAIAAoAE0ATgBfAGoAbQBUADIAMwAgACoAIAAoADEAIAAtACAARQBGAF8AbQBUADIAMwAgAC0AIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzACkAKQAgACoAIABQAEYAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBTAG8AaQBsAF8AcwBjAG8AcABlADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AOQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBTAG8AaQBsAF8AewBzAGMAbwBwAGUAMQB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAD0AMgAsADMAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgAsADMAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgAsADMAfQApACkAXABcAHQAaQBtAGUAcwAgAFAARgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAMgAzAFwAIgAsAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAGkAbgAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAYQBuAGQAIAB0AGUAcgB0AGkAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAcwB0AGEAZwBlAHMAIABhAHMAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIAA6ACAAawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AbQBUADIAMwBcACIALABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAZgBvAHIAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAZgBlAGUAZABsAG8AdAAgAGIAbwB1AG4AZABhAHIAeQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXABuAE0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAE0ATgBTAG8AaQBsAF8AcwBjAG8AcABlADMAXABuAGsAZwAgAE4AXABuAE0ATgBTAG8AaQBsAF8AewBzAGMAbwBwAGUAMwB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAD0AMgAsADMAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgAsADMAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgAsADMAfQApACkAXABcAHQAaQBtAGUAcwAoADEALQBQAEYAKQBcAG4ATQBOAF8AagBtAFQAMgAzACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAAcwBlAGMAbwBuAGQAYQByAHkAIABhAG4AZAAgAHQAZQByAHQAaQBhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAIABzAHQAYQBnAGUAcwAgAGEAcwAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAG8AcgAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgADoAIABrAGcAIABOAFwAbgBFAEYAXwBtAFQAMgAzACAAPQAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBhAGMAaAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXABuAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAZgBvAHIAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAbgBQAEYAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABmAGUAZQBkAGwAbwB0ACAAYgBvAHUAbgBkAGEAcgB5ACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAyADMALAAgAEUARgBfAG0AVAAyADMALAAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMALAAgAFAARgAsAFwAbgAgACAAIAAgACgATQBOAF8AagBtAFQAMgAzACAAKgAgACgAMQAgAC0AIABFAEYAXwBtAFQAMgAzACAALQAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMAKQApACAAKgAgACgAMQAgAC0AIABQAEYAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgA5ACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAzAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAPQAyACwAMwB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARQBGAF8AewBtAFQAPQAyACwAMwB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyACwAMwB9ACkAKQBcAFwAdABpAG0AZQBzACgAMQAtAFAARgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVAAyADMAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAAcwBlAGMAbwBuAGQAYQByAHkAIABhAG4AZAAgAHQAZQByAHQAaQBhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAIABzAHQAYQBnAGUAcwAgAGEAcwAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAG8AcgAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgADoAIABrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBtAFQAMgAzAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABhAG4AaQBtAGEAbAAgAHcAYQBzAHQAZQAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABpAG4AIABlAGEAYwBoACAATQBNAFMAIABmAG8AcgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABmAGUAZQBkAGwAbwB0ACAAYgBvAHUAbgBkAGEAcgB5ACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgAxADoAIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEALgAxAC4ANQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABNAGEAbgB1AHIAZQAgAEEAdABtAG8AcwBwAGgAZQByAGkAYwAgAEQAZQBwAG8AcwBpAHQAaQBvAG4AIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAYQB0AG0AbwBzAHAAaABlAHIAaQBjACAAZABlAHAAbwBzAGkAdABpAG8AbgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ARQBfAE4AMgBPAGEAZABcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGEAZAB9AD0AKABNAE0AUwBfAHsAQQBUAE0ATwBTAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcAG4ATQBNAFMAXwBBAFQATQBPAFMAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAIAA6ACAAawBnACAATgBcAG4ARQBGAF8ATgAyAE8AIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABhAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AQQBUAE0ATwBTACwAIABFAEYAXwBOADIATwAsACAAQwBfAE4AMgBPACwAXABuACAAIAAgACAAKABNAE0AUwBfAEEAVABNAE8AUwAgACoAIABFAEYAXwBOADIATwAgACoAIABDAF8ATgAyAE8AKQAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABhAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AYQBkAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABhAGQAfQA9ACgATQBNAFMAXwB7AEEAVABNAE8AUwB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBBAFQATQBPAFMAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAE0ATQBTACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAE4AMgBPAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAFwAIgAsACAAXAAiAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAIABuAGkAdAByAG8AZwBlAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBNAE0AUwBfAEEAVABNAE8AUwBcAG4AawBnACAATgBcAG4ATQBNAFMAXwB7AEEAVABNAE8AUwB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAH0AKQBcAG4ATQBOAF8AagBtAFQAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAATQBNAFMAIAAoAGUAeABjAGwAdQBkAGkAbgBnACAATQBOAF8AaQBqAG0AMQAzAFQAMgApACAAOgAgAGsAZwAgAE4AXABuAEYAcgBhAGMARwBBAFMATQBfAG0AVAAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAOgAgACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtAFQALAAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAsAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUACAAKgAgAEYAcgBhAGMARwBBAFMATQBfAG0AVABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBvAGwAYQB0AGkAbABpAHMAZQBkACAAbgBpAHQAcgBvAGcAZQBuACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBfAEEAVABNAE8AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAF8AewBBAFQATQBPAFMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEcAQQBTAE0AXwB7AG0AVAB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVABcACIALABcACIAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAATQBNAFMAIAAoAGUAeABjAGwAdQBkAGkAbgBnACAATQBOAF8AaQBqAG0AMQAzAFQAMgApACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBfAG0AVABcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEAOgAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4AMQAuADEALgAzACAATQBlAHQAaABvAGQAIAAxACAALQAgAE0AYQBuAHUAcgBlACAARABpAHIAZQBjAHQAIABOADIATwAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABkAGkAcgBlAGMAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQBzAFwAbgBFAF8ATgAyAE8AZABpAHIAXABuAHQAIABOADIATwBcAG4ARQBfAHsATgAyAE8ALABkAGkAcgB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAagBtAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXABuAE0ATgBfAGoAbQBUACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAALAAgAE0ATQBTACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADoAIABrAGcAIABOAFwAbgBFAEYAXwBqAG0AIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABNAE0AUwAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAbgBDAF8ATgAyAE8AIAA9ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwAgADoAIAByAGEAdABpAG8AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAsACAARQBGAF8AagBtACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgATQBOAF8AagBtAFQALAAgAEUARgBfAGoAbQAsACAAQwBfAE4AMgBPACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAZABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAE4AMgBPAGQAaQByAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABkAGkAcgB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAagBtAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAXAAiACwAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAALAAgAE0ATQBTACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADoAIABrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBqAG0AXAAiACwAXAAiAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAATQBNAFMAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXABuAE0ATgBfAGoAbQA1AFQAMQBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0APQA1ACwAVAA9ADEAfQA9AEEARQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtAD0ANQAsAFQAPQAxAH0AXABuAEEARQBfAGoAIAA9ACAAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGsAZwAgAE4AXABuAE0ATQBTAF8AagBtADUAVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQBFAF8AagAsACAATQBNAFMAXwBqAG0ANQBUADEALABcAG4AIAAgACAAIABBAEUAXwBqACAAKgAgAE0ATQBTAF8AagBtADUAVAAxAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtADUAVAAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AD0AQQBFAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0APQA1ACwAVAA9ADEAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAF8AagBcACIALABcACIAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AagBtADUAVAAxAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXABuAEEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAaQBvAG4AIABmAHIAbwBtACAAZQBhAGMAaAAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcABcAG4AQQBFAF8AagBcAG4AawBnACAATgBcAG4AQQBFAF8AewBqAH0APQBOAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE4ARQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAH0AXABuAE4AXwBqACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGgAZQBhAGQAXABuAE4ARQBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAaQBvAG4AIAA6ACAAawBnACAATgAvAGgAZQBhAGQALwBkAGEAeQBcAG4ARABfAGoAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGQAYQB5AHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATgBFAF8AagAsACAARABfAGoALABcAG4AIAAgACAAIABOAF8AagAgACoAIABOAEUAXwBqACAAKgAgAEQAXwBqAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBuAG4AdQBhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgAGYAcgBvAG0AIABlAGEAYwBoACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEUAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQBfAHsAagB9AD0ATgBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABOAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqAFwAIgAsAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABoAGUAYQBkAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEUAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgADoAIABrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagBcACIALABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGQAYQB5AHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAFwAbgBOAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgAHAAZQByACAAaABlAGEAZAAgAHAAZQByACAAZABhAHkAXABuAE4ARQBfAGoAXABuAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAE4ARQBfAHsAagB9AD0ATgBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAoADEALQBOAFIAXwB7AGoAfQApAFwAbgBOAEkAXwBqACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgB0AGEAawBlACAAOgAgAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAE4AUgBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAcgBlAHQAZQBuAHQAaQBvAG4AIABlAHgAcAByAGUAcwBzAGUAZAAgAGEAcwAgAGEAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABpAG4AdABhAGsAZQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4ASQBfAGoALAAgAE4AUgBfAGoALABcAG4AIAAgACAAIABOAEkAXwBqACAAKgAgACgAMQAgAC0AIABOAFIAXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuACAAcABlAHIAIABoAGUAYQBkACAAcABlAHIAIABkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEUAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBFAF8AewBqAH0APQBOAEkAXwB7AGoAfQBcAFwAdABpAG0AZQBzACgAMQAtAE4AUgBfAHsAagB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEkAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIABpAG4AdABhAGsAZQAgADoAIABrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFIAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIAByAGUAdABlAG4AdABpAG8AbgAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGkAbgB0AGEAawBlACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAFwAbgBOAGkAdAByAG8AZwBlAG4AIABpAG4AdABhAGsAZQAgAG8AZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQBcAG4ATgBJAF8AagBcAG4AawBnACAATgAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATgBJAF8AewBqAH0APQBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEMAUABfAHsAagB9AFwAXABkAGkAdgAgADYALgAyADUAXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABpAG4AdABhAGsAZQAgADoAIABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAEMAUABfAGoAIAA9ACAAYwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ANgAuADIANQAgAD0AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAYwBvAG4AdgBlAHIAdABpAG4AZwAgAGMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABpAG4AdABvACAAbgBpAHQAcgBvAGcAZQBuACAAOgAgAHIAYQB0AGkAbwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEkAXwBqACwAIABDAFAAXwBqACwAXABuACAAIAAgACAASQBfAGoAIAAqACAAQwBQAF8AagAgAC8AIAA2AC4AMgA1AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAaQBuAHQAYQBrAGUAIABvAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBJAF8AewBqAH0APQBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEMAUABfAHsAagB9AFwAXABkAGkAdgAgADYALgAyADUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABpAG4AdABhAGsAZQAgADoAIABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAUABfAGoAXAAiACwAXAAiAGMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiADYALgAyADUAXAAiACwAXAAiAGYAYQBjAHQAbwByACAAZgBvAHIAIABjAG8AbgB2AGUAcgB0AGkAbgBnACAAYwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGkAbgB0AG8AIABuAGkAdAByAG8AZwBlAG4AIAA6ACAAcgBhAHQAaQBvAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgBOAGkAdAByAG8AZwBlAG4AIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcAG4ATQBOAF8AagBtAFQAMgBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0ALABUAD0AMgB9AD0ATgBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtACwAVAA9ADIAfQBcAG4ATgBUAF8AagBtAFQAMgAgAD0AIABuAGkAdAByAG8AZwBlAG4AIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIABzAGUAYwBvAG4AZABhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAIAA6ACAAawBnACAATgBcAG4ATQBNAFMAXwBqAG0AVAAyACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAZQBhAGMAaAAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIALAAgAE0ATQBTAF8AagBtAFQAMgAsAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIAIAAqACAATQBNAFMAXwBqAG0AVAAyAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AewBqAG0ALABUAD0AMgB9AD0ATgBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtACwAVAA9ADIAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBUAF8AagBtAFQAMgBcACIALABcACIAbgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAcwBlAGMAbwBuAGQAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AagBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAFwAbgBOAGkAdAByAG8AZwBlAG4AIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcAG4ATgBUAF8AagBtAFQAMgBcAG4AawBnACAATgBcAG4ATgBUAF8AewBqAG0ALABUAD0AMgB9AD0AKABNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAD0ANQB9AC0ARQBGAF8AewBtAD0ANQB9ACkAKQAtAE0ATgBfAHsAagBtACwAVAA9ADMAfQBcAG4ATQBOAF8AagBtADUAVAAxACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAE0ATQBTACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAAOgAgAGsAZwAgAE4AXABuAEYAcgBhAGMARwBBAFMATQBfAG0ANQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBFAEYAXwBtADUAIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABkAGUAcABvAHMAaQB0AGUAZABcAG4ATQBOAF8AagBtAFQAMwAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABNAE0AUwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMwAgADoAIABrAGcAIABOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0ANQBUADEALAAgAEYAcgBhAGMARwBBAFMATQBfAG0ANQAsACAARQBGAF8AbQA1ACwAIABNAE4AXwBqAG0AVAAzACwAXABuACAAIAAgACAAKABNAE4AXwBqAG0ANQBUADEAIAAqACAAKAAxACAALQAgAEYAcgBhAGMARwBBAFMATQBfAG0ANQAgAC0AIABFAEYAXwBtADUAKQApACAALQAgAE0ATgBfAGoAbQBUADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AVABfAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADcAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAFQAXwB7AGoAbQAsAFQAPQAyAH0APQAoAE0ATgBfAHsAagBtAD0ANQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0APQA1AH0ALQBFAEYAXwB7AG0APQA1AH0AKQApAC0ATQBOAF8AewBqAG0ALABUAD0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtADUAVAAxAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIABpAG4AIABNAE0AUwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgADoAIABrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AXwBtADUAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAG0ANQBcACIALABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABkAGUAcABvAHMAaQB0AGUAZABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAMwBcACIALABcACIAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADMAIAA6ACAAawBnACAATgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAzACAATQBNAFMAXABuAE0ATgBfAGoAbQAxAFQAMwBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0APQAxACwAVAA9ADMAfQA9AEEARQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtAD0AMQAsAFQAPQAzAH0AXABuAEEARQBfAGoAIAA9ACAAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGsAZwAgAE4AXABuAE0ATQBTAF8AagBtADEAVAAzACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAdABvACAAdABlAHIAdABpAGEAcgB5ACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAEUAXwBqACwAIABNAE0AUwBfAGoAbQAxAFQAMwAsAFwAbgAgACAAIAAgAEEARQBfAGoAIAAqACAATQBNAFMAXwBqAG0AMQBUADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAzACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwBqAG0AMQBUADMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA4ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBfAHsAagBtAD0AMQAsAFQAPQAzAH0APQBBAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AGoAbQA9ADEALABUAD0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEUAXwBqAFwAIgAsAFwAIgB0AG8AdABhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABlAGQAIABiAHkAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0AMQBUADMAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAdABvACAAdABlAHIAdABpAGEAcgB5ACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4ACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAFIAZQBzAGkAZAB1AGUAQwByAG8AcABSAGEAdABpAG8AIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAFIAZQBzAGkAZAB1AGUAUgBlAG0AbwB2AGUAZAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADMATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATABpAHYAZQBzAHQAbwBjAGsAQwBsAGEAcwBzAGUAcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0AF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -27919,11 +27537,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAIgAsACIAdABlAHgAdAAiADoAIgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGwAbwBzAHQAIABpAG4AIAB0AGgAZQAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkAGwAbwB0ACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAFMATABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA1ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AG8AIABlAGEAYwBoACAAdABlAHIAdABpAGEAcgB5ACAAcwB5AHMAdABlAG0AIABhAHMAcwB1AG0AZQBkACAAdABoAGEAdAAgADIAIABwAGUAcgAgAGMAZQBuAHQAIABpAHMAIAByAHUAbgAgAC0AIABvAGYAZgAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAZQBlAGQAIABwAGEAZAAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AG8AIABlAGEAYwBoACAAdABlAHIAdABpAGEAcgB5ACAAcwB5AHMAdABlAG0AIABhAHMAcwB1AG0AZQBkACAAdABoAGEAdAAgADIAIABwAGUAcgAgAGMAZQBuAHQAIABpAHMAIAByAHUAbgAgAC0AIABvAGYAZgAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAZQBlAGQAIABwAGEAZAAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAG0AMQBUADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AFwAbgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA2ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4ATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBtADMAIABDAEgANAAgAC8AIABrAGcAIABWAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA5ACkAOwBcAG4AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAxAE0ATQBTAE8AcAB0AGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAE0ATQBTAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBTAHQAYQBnAGUAMwBNAE0AUwBPAHAAdABpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBMAGkAdgBlAHMAdABvAGMAawBDAGwAYQBzAHMAZQBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQB4AHAAbwByAHQAIABtAGkAZAAgAGYAZQBkAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAeABwAG8AcgB0ACAAbABvAG4AZwAgAGYAZQBkAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgAxADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIAAoAGQAYQB5AHMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAKABkAGEAeQBzACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADEAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgACgAZABhAHkAcwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIATABlAG4AZwB0AGgAIABvAGYAIABTAHQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIAMQAtADgAMAAgAGQAYQB5AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIAOAAxAC0AMgAwADAAIABkAGEAeQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIAMgAwADEAKwAgAGQAYQB5AHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADIAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEEAbgBpAG0AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgAyADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEEAbgBpAG0AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAHYAZQBkACAAZgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAcwAgAHQAbwAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBhAG0AZQBkACAAXAB1ADAAMAAyADcAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAAtACAAbwByAGkAZwBpAG4AYQBsACAAaABhAHMAIABoAGUAYQBkAGUAcgAgAFwAdQAwADAAMgA3AFUAbgBpAHQAXAB1ADAAMAAyADcAIAB3AGgAaQBjAGgAIABjAG8AdgBlAHIAcwAgAHQAdwBvACAAYwBvAGwAdQBtAG4AcwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADAALAAgADcALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBlAGQAbABvAHQAIAB0AHkAcABlAFwAIgAsACAAXAAiAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBcACIALAAgAFwAIgBVAG4AaQB0AFwAIgAsACAAXAAiADIAMAAwADUALQAyADAAMAA5AFwAIgAsACAAXAAiADIAMAAxADAALQAyADAAMQA0AFwAIgAsACAAXAAiADIAMAAxADUALQAyADAAMQA5AFwAIgAsACAAXAAiADIAMAAyADAALQAyADAAMgAzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARABhAHkAcwAgAG8AbgAgAGYAZQBlAGQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgADcAMAAsACAANwAwACwAIAA3ADAALAAgADcANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAMQAwAC4AMAAsACAAMQAwAC4AMAAsACAAMQAwAC4ANAAsACAAMQAwAC4ANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIATgAgAHIAZQB0AGUAbgB0AGkAbwBuAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdAAgAG8AZgAgAGkAbgB0AGEAawBlAFwAIgAsACAAMgAxAC4AMQAsACAAMgAwAC4ANAAsACAAMgAwAC4ANAAsACAAMgAwAC4ANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEQAYQB5AHMAIABvAG4AIABmAGUAZQBkAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIAAxADEANQAsACAAMQAxADUALAAgADEAMgAwACwAIAAxADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBkAGEAeQBcACIALAAgADEAMQAuADIALAAgADEAMAAuADgALAAgADEAMAAuADgALAAgADEAMAAuADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBOACAAcgBlAHQAZQBuAHQAaQBvAG4AXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0ACAAbwBmACAAaQBuAHQAYQBrAGUAXAAiACwAIAAxADIALgA1ACwAIAAxADIALgA3ACwAIAAxADIALgA3ACwAIAAxADIALgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgBEAGEAeQBzACAAbwBuACAAZgBlAGUAZABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAMgA1ADAALAAgADIANQAwACwAIAAyADUAMAAsACAAMgA1ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBkAGEAeQBcACIALAAgADkALgAwACwAIAA4AC4ANQAsACAAOAAuADIALAAgADgALgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgBOACAAcgBlAHQAZQBuAHQAaQBvAG4AXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0ACAAbwBmACAAaQBuAHQAYQBrAGUAXAAiACwAIAA2AC4ANgAsACAANwAuADAALAAgADcALgAwACwAIAA3AC4AMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADMAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARABpAGUAdAAgAHAAcgBvAHAAZQByAHQAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARABpAGUAdAAgAHAAcgBvAHAAZQByAHQAaQBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADMAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARABpAGUAdAAgAHAAcgBvAHAAZQByAHQAaQBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AEMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAZgByAGEAYwB0AGkAbwBuACAAYwBvAGwAdQBtAG4AIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAATgBEAEYAIABhAG4AZAAgAEUAdABoAGUAcgAgAGUAeAB0AHIAYQBjAHQAIAB2AGEAbAB1AGUAcwAgAHQAbwAgAGYAcgBhAGMAdABpAG8AbgBzAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwB2AGUAZAAgAGYAZQBlAGQAbABvAHQAIAB0AHkAcABlAHMAIAB0AG8AIABhACAAcwBlAHAAYQByAGEAdABlACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADgALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBlAGQAbABvAHQAIAB0AHkAcABlAFwAIgAsACAAXAAiAE4AdQB0AHIAaQBlAG4AdAAgAGEAbgBhAGwAeQBzAGkAcwBcACIALAAgAFwAIgBVAG4AaQB0AFwAIgAsACAAXAAiADIAMAAwADUALQAyADAAMAA5AFwAIgAsACAAXAAiADIAMAAxADAALQAyADAAMQA0AFwAIgAsACAAXAAiADIAMAAxADUALQAyADAAMQA5AFwAIgAsACAAXAAiADIAMAAyADAALQAyADAAMgAzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAZgByAGEAYwB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBOAEQARgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAAyADMALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAwAC4AMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBFAHQAaABlAHIAIABFAHgAdAByAGEAYwB0AFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADQALgA1ACwAIAA0AC4ANQAsACAANAAuADgALAAgADQALgA4ACwAIAAwAC4AMAA0ADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQAzACwAIAAwAC4AMQAyADUALAAgADAALgAxADIALAAgADAALgAxADIALAAgADAALgAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBOAEQARgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAAyADQALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAwAC4AMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARQB0AGgAZQByACAARQB4AHQAcgBhAGMAdABcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAA1AC4AMAAsACAANQAuADAALAAgADUALgAwACwAIAA1AC4AMAAsACAAMAAuADAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQAzACwAIAAwAC4AMQAyADUALAAgADAALgAxADIALAAgADAALgAxADIALAAgADAALgAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAE4ARABGAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADIANAAuADAALAAgADIANAAuADAALAAgADIANAAuADAALAAgADIANAAuADAALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAEUAdABoAGUAcgAgAEUAeAB0AHIAYQBjAHQAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAANQAuADAALAAgADUALgAwACwAIAA1AC4ANQAsACAANQAuADUALAAgADAALgAwADUANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADQAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQBUACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABNAEMARgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANAA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHUAcABsAGkAYwBhAHQAZQBkACAATgBTAFcAIAB2AGEAbAB1AGUAcwAgAGYAbwByACAAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAE4AVAAgAGEAbgBkACAAVABBAFMAIABjAG8AbAB1AG0AbgBzACAAdwBpAHQAaAAgAFwAdQAwADAAMgA3AG4AbwAgAGQAYQB0AGEAXAB1ADAAMAAyADcAIAB2AGEAbAB1AGUAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMQAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAE4AUwBXAFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAE4AVABcACIALAAgAFwAIgBTAEEAXAAiACwAIABcACIAVgBJAEMAXAAiACwAIABcACIAVwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAzACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBOAG8AIABkAGEAdABhAFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlACAAKABTAHQAbwBjAGsAcABpAGwAZQApAFwAIgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAXAAiAE4AbwAgAGQAYQB0AGEAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBOAG8AIABkAGEAdABhAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAMAAsACAAMAAsACAAXAAiAE4AbwAgAGQAYQB0AGEAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAcgB0AGkAYQByAHkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAKABFAGYAZgBsAHUAZQBuAHQAIABwAG8AbgBkACkAXAAiACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA3ACwAIABcACIATgBvACAAZABhAHQAYQBcACIALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgAFwAIgBOAG8AIABkAGEAdABhAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADUAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzACAAKABFAEYAbQBUACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgA1ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgACgARQBGAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAE0ATQBTACAAbgBhAG0AZQBzACAAdABoAGEAdAAgAG0AYQB0AGMAaAAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAVABcACIALAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AVAAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4AMAAwADUANAAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQAgACgAUwB0AG8AYwBrAHAAaQBsAGUAKQBcACIALAAgADAALgAwADAANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4AMAAxACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAcgB0AGkAYQByAHkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAKABFAGYAZgBsAHUAZQBuAHQAIABQAG8AbgBkACkAXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgA2ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwAgACgARgByAGEAYwBHAEEAUwBNAG0AVAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgA2ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwAgACgARgByAGEAYwBHAEEAUwBNAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEYAcgBhAGMARwBBAFMATQBtAFQAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAaQBtAGEAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAbABvAHQAIAAoAEYAZQBlAGQAcABhAGQAKQBcACIALAAgADAALgA2ACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlACAAKABTAHQAbwBjAGsAcABpAGwAZQApAFwAIgAsACAAMAAuADIANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4ANAAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAHIAdABpAGEAcgB5AFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAApAFwAIgAsACAAMAAuADMANQAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEAOgAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4AMQAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAE0AYQBuAHUAcgBlACAATQBlAHQAaABhAG4AZQAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAXwBDAEgANABcAG4AdAAgAEMASAA0AFwAbgB7AEUAfQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgARABfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABOAF8AewBqAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXABuAEQAXwBqACAAPQAgAGwAZQBuAGcAdABoACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIABkAGEAeQBzAFwAbgBNAF8AagBtAFQAIAA9ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABwAGUAcgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACwAIABNAE0AUwAsACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADoAIABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAaABlAGEAZABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABfAGoALAAgAE0AXwBqAG0AVAAsACAATgBfAGoALABcAG4AIAAgACAAIAAoAEQAXwBqACAAKgAgAE0AXwBqAG0AVAAgACoAIABOAF8AagApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAEgANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHsARQB9AF8AewBDAEgANAB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABEAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAE4AXwB7AGoAfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqAFwAIgAsAFwAIgBsAGUAbgBnAHQAaAAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAZABhAHkAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAbQBUAFwAIgAsAFwAIgBtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAHAAZQByACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAALAAgAE0ATQBTACwAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAOgAgAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALABcACIAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAaABlAGEAZABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AFwAbgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAE0ATQBTAFwAbgBNAF8AagBtADUAVAAxAFwAbgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBfAHsAagBtAD0ANQAsAFQAPQAxAH0APQBWAFMAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAAQgBPAFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAD0ANQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXABuAFYAUwBfAGoAIAA9ACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4AQgBPACAAPQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAIAA6ACAAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXABuAE0ATQBTAF8AbQA1AFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBNAEMARgBfAGkAbQA1ACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGQAcgB5AGwAbwB0ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAFMAXwBqACwAIABCAE8ALAAgAE0ATQBTAF8AbQA1AFQAMQAsACAATQBDAEYAXwBpAG0ANQAsACAAcgBoAG8ALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIABNAEMARgBfAGkAbQA1ACwAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABNAEMARgBfAGkAbQA1ACkALAAgAE0AQwBGAF8AaQBtADUALAAgADAAKQAsAFwAbgAgACAAIAAgACAAIABWAFMAXwBqACAAKgAgAEIATwAgACoAIABNAE0AUwBfAG0ANQBUADEAIAAqACAATQBDAEYAXwBpAG0ANQAgACoAIAByAGgAbwBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAbQA1AFQAMQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAagBtAD0ANQAsAFQAPQAxAH0APQBWAFMAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAAQgBPAFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAD0ANQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAG0ANQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtADUAXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGQAcgB5AGwAbwB0ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAGgAbwBcACIALABcACIAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAA6ACAAawBnAC8AbQAzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAFwAIgAsACAAXAAiAHMAdABhAHQAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAbgBNAF8AagBtAFQAMgBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGoAbQBUAD0AMgB9AD0AKAAxAC0AVgBTAEwAKQBcAFwAdABpAG0AZQBzACAAVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXABuAFYAUwBMACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AVgBTAF8AagAgAD0AIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBCAE8AIAA9ACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgADoAIABtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcAG4ATQBNAFMAXwBtAFQAMgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ATQBDAEYAXwBpAG0AIAA9ACAAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgAGEAbgBkACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAFMATAAsACAAVgBTAF8AagAsACAAQgBPACwAIABNAE0AUwBfAG0AVAAyACwAIABNAEMARgBfAGkAbQAsACAAcgBoAG8ALABcAG4AIAAgACAAIAAoADEAIAAtACAAVgBTAEwAKQAgACoAIABWAFMAXwBqACAAKgAgAEIATwAgACoAIABNAE0AUwBfAG0AVAAyACAAKgAgAE0AQwBGAF8AaQBtACAAKgAgAHIAaABvAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGoAbQBUAD0AMgB9AD0AKAAxAC0AVgBTAEwAKQBcAFwAdABpAG0AZQBzACAAVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAEwAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAG0AVAAyAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBDAEYAXwBpAG0AXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAE0ATQBTACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAOgAgAGsAZwAvAG0AMwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAaQBcACIALAAgAFwAIgBzAHQAYQB0AGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBcAG4AUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADMAIABNAE0AUwBcAG4ATQBfAGoAbQAxAFQAMwBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGoAbQA9ADEALABUAD0AMwB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0APQAxACwAVAA9ADMAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQA9ADEAfQBcAFwAdABpAG0AZQBzACAAXABcAHIAaABvAFwAbgBWAFMAXwBqACAAPQAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAEIATwAgAD0AIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAbgBNAE0AUwBfAG0AMQBUADMAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIAB0AG8AIAB0AGUAcgB0AGkAYQByAHkAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBNAEMARgBfAGkAbQAxACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAHIAaABvACAAPQAgAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlACAAOgAgAGsAZwAvAG0AMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAUwBfAGoALAAgAEIATwAsACAATQBNAFMAXwBtADEAVAAzACwAIABNAEMARgBfAGkAbQAxACwAIAByAGgAbwAsAFwAbgAgACAAIAAgAFYAUwBfAGoAIAAqACAAQgBPACAAKgAgAE0ATQBTAF8AbQAxAFQAMwAgACoAIABNAEMARgBfAGkAbQAxACAAKgAgAHIAaABvAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADMAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAbQAxAFQAMwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANAApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAagBtAD0AMQAsAFQAPQAzAH0APQBWAFMAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAAQgBPAFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAbQA9ADEALABUAD0AMwB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAagAgADoAIABrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIATwBcACIALABcACIAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgADoAIABtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBtADEAVAAzAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAHQAbwAgAHQAZQByAHQAaQBhAHIAeQAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtADEAXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsAFwAIgBkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAFYAUwBfAGoAXABuAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4AVgBTAF8AewBqAH0APQBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAoADEALQBEAE0ARABfAHsAagB9ACkAXABcAHQAaQBtAGUAcwAoADEALQBBACkAXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABpAG4AdABhAGsAZQAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAEQATQBEAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAEEAIAA9ACAAYQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALAAgAEQATQBEAF8AagAsACAAQQAsAFwAbgAgACAAIAAgAEkAXwBqACAAKgAgACgAMQAgAC0AIABEAE0ARABfAGoAKQAgACoAIAAoADEAIAAtACAAQQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBTAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBfAHsAagB9AD0ASQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARABNAEQAXwB7AGoAfQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AQQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAXwBqAFwAIgAsAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIABqACAAOgAgAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgAGoAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAFwAIgAsAFwAIgBhAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgAxADoAIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEALgAxAC4AOQAgAE0AYQBuAHUAcgBlACAAQQBwAHAAbABpAGUAZAAgAHQAbwAgAFMAbwBpAGwAcwBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAxAFwAbgBrAGcAIABOAFwAbgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADEAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAA9ADIALAAzAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIALAAzAH0ALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0AVAA9ADIALAAzAH0AKQApAFwAXAB0AGkAbQBlAHMAIABQAEYAXABuAE0ATgBfAGoAbQBUADIAMwAgAD0AIABtAGEAcwBzACAAbwBmACAATgAgAGkAbgAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAYQBuAGQAIAB0AGUAcgB0AGkAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAcwB0AGEAZwBlAHMAIABhAHMAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIAA6ACAAawBnACAATgBcAG4ARQBGAF8AbQBUADIAMwAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAbgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGEAbgBpAG0AYQBsACAAdwBhAHMAdABlACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgAGYAbwByACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcAG4AUABGACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAZgBlAGUAZABsAG8AdAAgAGIAbwB1AG4AZABhAHIAeQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtAFQAMgAzACwAIABFAEYAXwBtAFQAMgAzACwAIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzACwAIABQAEYALABcAG4AIAAgACAAIAAoAE0ATgBfAGoAbQBUADIAMwAgACoAIAAoADEAIAAtACAARQBGAF8AbQBUADIAMwAgAC0AIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzACkAKQAgACoAIABQAEYAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBTAG8AaQBsAF8AcwBjAG8AcABlADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AOQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBTAG8AaQBsAF8AewBzAGMAbwBwAGUAMQB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAD0AMgAsADMAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgAsADMAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgAsADMAfQApACkAXABcAHQAaQBtAGUAcwAgAFAARgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAMgAzAFwAIgAsAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAGkAbgAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAYQBuAGQAIAB0AGUAcgB0AGkAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAcwB0AGEAZwBlAHMAIABhAHMAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIAA6ACAAawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AbQBUADIAMwBcACIALABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAZgBvAHIAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAZgBlAGUAZABsAG8AdAAgAGIAbwB1AG4AZABhAHIAeQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXABuAE0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAE0ATgBTAG8AaQBsAF8AcwBjAG8AcABlADMAXABuAGsAZwAgAE4AXABuAE0ATgBTAG8AaQBsAF8AewBzAGMAbwBwAGUAMwB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAD0AMgAsADMAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgAsADMAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgAsADMAfQApACkAXABcAHQAaQBtAGUAcwAoADEALQBQAEYAKQBcAG4ATQBOAF8AagBtAFQAMgAzACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAAcwBlAGMAbwBuAGQAYQByAHkAIABhAG4AZAAgAHQAZQByAHQAaQBhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAIABzAHQAYQBnAGUAcwAgAGEAcwAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAG8AcgAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgADoAIABrAGcAIABOAFwAbgBFAEYAXwBtAFQAMgAzACAAPQAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBhAGMAaAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXABuAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAZgBvAHIAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAbgBQAEYAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABmAGUAZQBkAGwAbwB0ACAAYgBvAHUAbgBkAGEAcgB5ACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAyADMALAAgAEUARgBfAG0AVAAyADMALAAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMALAAgAFAARgAsAFwAbgAgACAAIAAgACgATQBOAF8AagBtAFQAMgAzACAAKgAgACgAMQAgAC0AIABFAEYAXwBtAFQAMgAzACAALQAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMAKQApACAAKgAgACgAMQAgAC0AIABQAEYAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgA5ACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAzAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAPQAyACwAMwB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARQBGAF8AewBtAFQAPQAyACwAMwB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyACwAMwB9ACkAKQBcAFwAdABpAG0AZQBzACgAMQAtAFAARgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVAAyADMAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAAcwBlAGMAbwBuAGQAYQByAHkAIABhAG4AZAAgAHQAZQByAHQAaQBhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAIABzAHQAYQBnAGUAcwAgAGEAcwAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAG8AcgAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgADoAIABrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBtAFQAMgAzAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAzAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABhAG4AaQBtAGEAbAAgAHcAYQBzAHQAZQAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABpAG4AIABlAGEAYwBoACAATQBNAFMAIABmAG8AcgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABmAGUAZQBkAGwAbwB0ACAAYgBvAHUAbgBkAGEAcgB5ACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgAxADoAIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEALgAxAC4ANQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABNAGEAbgB1AHIAZQAgAEEAdABtAG8AcwBwAGgAZQByAGkAYwAgAEQAZQBwAG8AcwBpAHQAaQBvAG4AIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAYQB0AG0AbwBzAHAAaABlAHIAaQBjACAAZABlAHAAbwBzAGkAdABpAG8AbgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ARQBfAE4AMgBPAGEAZABcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGEAZAB9AD0AKABNAE0AUwBfAHsAQQBUAE0ATwBTAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcAG4ATQBNAFMAXwBBAFQATQBPAFMAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAIAA6ACAAawBnACAATgBcAG4ARQBGAF8ATgAyAE8AIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABhAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AQQBUAE0ATwBTACwAIABFAEYAXwBOADIATwAsACAAQwBfAE4AMgBPACwAXABuACAAIAAgACAAKABNAE0AUwBfAEEAVABNAE8AUwAgACoAIABFAEYAXwBOADIATwAgACoAIABDAF8ATgAyAE8AKQAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABhAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AYQBkAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABhAGQAfQA9ACgATQBNAFMAXwB7AEEAVABNAE8AUwB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBBAFQATQBPAFMAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAE0ATQBTACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAE4AMgBPAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAFwAIgAsACAAXAAiAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAIABuAGkAdAByAG8AZwBlAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBNAE0AUwBfAEEAVABNAE8AUwBcAG4AawBnACAATgBcAG4ATQBNAFMAXwB7AEEAVABNAE8AUwB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAH0AKQBcAG4ATQBOAF8AagBtAFQAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAATQBNAFMAIAAoAGUAeABjAGwAdQBkAGkAbgBnACAATQBOAF8AaQBqAG0AMQAzAFQAMgApACAAOgAgAGsAZwAgAE4AXABuAEYAcgBhAGMARwBBAFMATQBfAG0AVAAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAOgAgACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtAFQALAAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAsAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUACAAKgAgAEYAcgBhAGMARwBBAFMATQBfAG0AVABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBvAGwAYQB0AGkAbABpAHMAZQBkACAAbgBpAHQAcgBvAGcAZQBuACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBfAEEAVABNAE8AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAF8AewBBAFQATQBPAFMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEcAQQBTAE0AXwB7AG0AVAB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVABcACIALABcACIAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAATQBNAFMAIAAoAGUAeABjAGwAdQBkAGkAbgBnACAATQBOAF8AaQBqAG0AMQAzAFQAMgApACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBfAG0AVABcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEAOgAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4AMQAuADEALgAzACAATQBlAHQAaABvAGQAIAAxACAALQAgAE0AYQBuAHUAcgBlACAARABpAHIAZQBjAHQAIABOADIATwAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABkAGkAcgBlAGMAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQBzAFwAbgBFAF8ATgAyAE8AZABpAHIAXABuAHQAIABOADIATwBcAG4ARQBfAHsATgAyAE8ALABkAGkAcgB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAagBtAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXABuAE0ATgBfAGoAbQBUACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAALAAgAE0ATQBTACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADoAIABrAGcAIABOAFwAbgBFAEYAXwBqAG0AIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABNAE0AUwAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAbgBDAF8ATgAyAE8AIAA9ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwAgADoAIAByAGEAdABpAG8AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAsACAARQBGAF8AagBtACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgATQBOAF8AagBtAFQALAAgAEUARgBfAGoAbQAsACAAQwBfAE4AMgBPACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAZABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAE4AMgBPAGQAaQByAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABkAGkAcgB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABNAE4AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAagBtAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAXAAiACwAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAALAAgAE0ATQBTACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADoAIABrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBqAG0AXAAiACwAXAAiAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAATQBNAFMAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXABuAE0ATgBfAGoAbQA1AFQAMQBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0APQA1ACwAVAA9ADEAfQA9AEEARQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtAD0ANQAsAFQAPQAxAH0AXABuAEEARQBfAGoAIAA9ACAAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGsAZwAgAE4AXABuAE0ATQBTAF8AagBtADUAVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQBFAF8AagAsACAATQBNAFMAXwBqAG0ANQBUADEALABcAG4AIAAgACAAIABBAEUAXwBqACAAKgAgAE0ATQBTAF8AagBtADUAVAAxAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtADUAVAAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AD0AQQBFAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0APQA1ACwAVAA9ADEAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAF8AagBcACIALABcACIAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AagBtADUAVAAxAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXABuAEEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAaQBvAG4AIABmAHIAbwBtACAAZQBhAGMAaAAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcABcAG4AQQBFAF8AagBcAG4AawBnACAATgBcAG4AQQBFAF8AewBqAH0APQBOAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE4ARQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAH0AXABuAE4AXwBqACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGgAZQBhAGQAXABuAE4ARQBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAaQBvAG4AIAA6ACAAawBnACAATgAvAGgAZQBhAGQALwBkAGEAeQBcAG4ARABfAGoAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGQAYQB5AHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATgBFAF8AagAsACAARABfAGoALABcAG4AIAAgACAAIABOAF8AagAgACoAIABOAEUAXwBqACAAKgAgAEQAXwBqAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBuAG4AdQBhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgAGYAcgBvAG0AIABlAGEAYwBoACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEUAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQBfAHsAagB9AD0ATgBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABOAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqAFwAIgAsAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABoAGUAYQBkAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEUAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgADoAIABrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagBcACIALABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGQAYQB5AHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAFwAbgBOAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgAHAAZQByACAAaABlAGEAZAAgAHAAZQByACAAZABhAHkAXABuAE4ARQBfAGoAXABuAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAE4ARQBfAHsAagB9AD0ATgBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAoADEALQBOAFIAXwB7AGoAfQApAFwAbgBOAEkAXwBqACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgB0AGEAawBlACAAOgAgAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAE4AUgBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAcgBlAHQAZQBuAHQAaQBvAG4AIABlAHgAcAByAGUAcwBzAGUAZAAgAGEAcwAgAGEAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABpAG4AdABhAGsAZQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4ASQBfAGoALAAgAE4AUgBfAGoALABcAG4AIAAgACAAIABOAEkAXwBqACAAKgAgACgAMQAgAC0AIABOAFIAXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuACAAcABlAHIAIABoAGUAYQBkACAAcABlAHIAIABkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEUAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBFAF8AewBqAH0APQBOAEkAXwB7AGoAfQBcAFwAdABpAG0AZQBzACgAMQAtAE4AUgBfAHsAagB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEkAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIABpAG4AdABhAGsAZQAgADoAIABrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFIAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIAByAGUAdABlAG4AdABpAG8AbgAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGkAbgB0AGEAawBlACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAFwAbgBOAGkAdAByAG8AZwBlAG4AIABpAG4AdABhAGsAZQAgAG8AZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQBcAG4ATgBJAF8AagBcAG4AawBnACAATgAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATgBJAF8AewBqAH0APQBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEMAUABfAHsAagB9AFwAXABkAGkAdgAgADYALgAyADUAXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABpAG4AdABhAGsAZQAgADoAIABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAEMAUABfAGoAIAA9ACAAYwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ANgAuADIANQAgAD0AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAYwBvAG4AdgBlAHIAdABpAG4AZwAgAGMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABpAG4AdABvACAAbgBpAHQAcgBvAGcAZQBuACAAOgAgAHIAYQB0AGkAbwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEkAXwBqACwAIABDAFAAXwBqACwAXABuACAAIAAgACAASQBfAGoAIAAqACAAQwBQAF8AagAgAC8AIAA2AC4AMgA1AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAaQBuAHQAYQBrAGUAIABvAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBJAF8AewBqAH0APQBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEMAUABfAHsAagB9AFwAXABkAGkAdgAgADYALgAyADUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABpAG4AdABhAGsAZQAgADoAIABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAUABfAGoAXAAiACwAXAAiAGMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiADYALgAyADUAXAAiACwAXAAiAGYAYQBjAHQAbwByACAAZgBvAHIAIABjAG8AbgB2AGUAcgB0AGkAbgBnACAAYwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGkAbgB0AG8AIABuAGkAdAByAG8AZwBlAG4AIAA6ACAAcgBhAHQAaQBvAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgBOAGkAdAByAG8AZwBlAG4AIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcAG4ATQBOAF8AagBtAFQAMgBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0ALABUAD0AMgB9AD0ATgBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtACwAVAA9ADIAfQBcAG4ATgBUAF8AagBtAFQAMgAgAD0AIABuAGkAdAByAG8AZwBlAG4AIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIABzAGUAYwBvAG4AZABhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAIAA6ACAAawBnACAATgBcAG4ATQBNAFMAXwBqAG0AVAAyACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAZQBhAGMAaAAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIALAAgAE0ATQBTAF8AagBtAFQAMgAsAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIAIAAqACAATQBNAFMAXwBqAG0AVAAyAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AewBqAG0ALABUAD0AMgB9AD0ATgBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtACwAVAA9ADIAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBUAF8AagBtAFQAMgBcACIALABcACIAbgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAcwBlAGMAbwBuAGQAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AagBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAFwAbgBOAGkAdAByAG8AZwBlAG4AIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcAG4ATgBUAF8AagBtAFQAMgBcAG4AawBnACAATgBcAG4ATgBUAF8AewBqAG0ALABUAD0AMgB9AD0AKABNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAD0ANQB9AC0ARQBGAF8AewBtAD0ANQB9ACkAKQAtAE0ATgBfAHsAagBtACwAVAA9ADMAfQBcAG4ATQBOAF8AagBtADUAVAAxACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAE0ATQBTACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAAOgAgAGsAZwAgAE4AXABuAEYAcgBhAGMARwBBAFMATQBfAG0ANQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBFAEYAXwBtADUAIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABkAGUAcABvAHMAaQB0AGUAZABcAG4ATQBOAF8AagBtAFQAMwAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABNAE0AUwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMwAgADoAIABrAGcAIABOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0ANQBUADEALAAgAEYAcgBhAGMARwBBAFMATQBfAG0ANQAsACAARQBGAF8AbQA1ACwAIABNAE4AXwBqAG0AVAAzACwAXABuACAAIAAgACAAKABNAE4AXwBqAG0ANQBUADEAIAAqACAAKAAxACAALQAgAEYAcgBhAGMARwBBAFMATQBfAG0ANQAgAC0AIABFAEYAXwBtADUAKQApACAALQAgAE0ATgBfAGoAbQBUADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AVABfAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADcAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAFQAXwB7AGoAbQAsAFQAPQAyAH0APQAoAE0ATgBfAHsAagBtAD0ANQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0APQA1AH0ALQBFAEYAXwB7AG0APQA1AH0AKQApAC0ATQBOAF8AewBqAG0ALABUAD0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtADUAVAAxAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIABpAG4AIABNAE0AUwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgADoAIABrAGcAIABOAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AXwBtADUAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAG0ANQBcACIALABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABkAGUAcABvAHMAaQB0AGUAZABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAMwBcACIALABcACIAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADMAIAA6ACAAawBnACAATgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAzACAATQBNAFMAXABuAE0ATgBfAGoAbQAxAFQAMwBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0APQAxACwAVAA9ADMAfQA9AEEARQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtAD0AMQAsAFQAPQAzAH0AXABuAEEARQBfAGoAIAA9ACAAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGsAZwAgAE4AXABuAE0ATQBTAF8AagBtADEAVAAzACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAdABvACAAdABlAHIAdABpAGEAcgB5ACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAEUAXwBqACwAIABNAE0AUwBfAGoAbQAxAFQAMwAsAFwAbgAgACAAIAAgAEEARQBfAGoAIAAqACAATQBNAFMAXwBqAG0AMQBUADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAzACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwBqAG0AMQBUADMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA4ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBfAHsAagBtAD0AMQAsAFQAPQAzAH0APQBBAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AGoAbQA9ADEALABUAD0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEUAXwBqAFwAIgAsAFwAIgB0AG8AdABhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABlAGQAIABiAHkAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAIAA6ACAAawBnACAATgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0AMQBUADMAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAdABvACAAdABlAHIAdABpAGEAcgB5ACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4ACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAFIAZQBzAGkAZAB1AGUAQwByAG8AcABSAGEAdABpAG8AIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAFIAZQBzAGkAZAB1AGUAUgBlAG0AbwB2AGUAZAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADMATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATABpAHYAZQBzAHQAbwBjAGsAQwBsAGEAcwBzAGUAcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0AF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27942,15 +27564,15 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -27959,12 +27581,4 @@
     <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>